<commit_message>
feat(model): establish Star Schema topology and bridge table logic
Configured 1:N relationships for core dimensions and enabled bi-directional filtering on kpi_owners and kpi_sources to support Many-to-Many mapping.
</commit_message>
<xml_diff>
--- a/Datasets/okrs.xlsx
+++ b/Datasets/okrs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauro\Desktop\Accenture\Dashboard okrs\Datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2DA32F03-7B3A-48B6-86A3-0C7039136D37}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B4B868A1-57F6-4522-B5FD-356BC4675FBA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="810" activeTab="7" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="810" activeTab="3" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
   </bookViews>
   <sheets>
     <sheet name="objetives" sheetId="11" r:id="rId1"/>
@@ -1296,7 +1296,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="31">
+  <fonts count="32">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1489,6 +1489,14 @@
       <color rgb="FF464FEB"/>
       <name val="Segoe UI"/>
       <family val="2"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <color theme="0"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -1706,7 +1714,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="101">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1971,12 +1979,55 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="24">
+  <dxfs count="26">
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="12"/>
+        <color theme="0"/>
+        <name val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor theme="4"/>
+          <bgColor theme="4"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <border outline="0">
+        <left style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </left>
+        <right style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </right>
+        <top style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </top>
+        <bottom style="thin">
+          <color theme="4" tint="0.39997558519241921"/>
+        </bottom>
+      </border>
+    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -3005,11 +3056,11 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{656EB1B5-23C9-4E3F-9012-15F13CF03D91}" name="units" displayName="units" ref="A1:B3" totalsRowShown="0">
-  <autoFilter ref="A1:B3" xr:uid="{656EB1B5-23C9-4E3F-9012-15F13CF03D91}"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6AAE90B7-0747-44B6-892C-5C0FB09C6261}" name="units" displayName="units" ref="A1:B3" totalsRowShown="0" headerRowDxfId="0" tableBorderDxfId="1">
+  <autoFilter ref="A1:B3" xr:uid="{6AAE90B7-0747-44B6-892C-5C0FB09C6261}"/>
   <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{BB49761B-334A-4008-94DE-742BEE03B1C8}" name="Unit_ID"/>
-    <tableColumn id="2" xr3:uid="{07D21854-2CFA-4EFD-B6A7-7D9755E7A3C1}" name="Unit_Name"/>
+    <tableColumn id="1" xr3:uid="{78A9EFFF-8B69-456A-BE78-36EE4A6917F7}" name="Unit_ID"/>
+    <tableColumn id="2" xr3:uid="{AC9CF5AF-7CCA-440B-9A30-C4372D1D43D7}" name="Unit_Name"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3057,7 +3108,7 @@
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{D2F6C869-298A-4690-A078-35A0D201E072}" name="Result_ID"/>
     <tableColumn id="2" xr3:uid="{3F7B7E26-AE5E-4B25-BEF0-6F64A9729CC1}" name="KPI_ID"/>
-    <tableColumn id="3" xr3:uid="{1AEA6639-430E-4250-A1EC-1DCF4FC5151B}" name="Date" dataDxfId="23"/>
+    <tableColumn id="3" xr3:uid="{1AEA6639-430E-4250-A1EC-1DCF4FC5151B}" name="Date" dataDxfId="25"/>
     <tableColumn id="4" xr3:uid="{96F10FB5-5453-4273-8C7D-2EB9CF434694}" name="Actual_Value"/>
     <tableColumn id="5" xr3:uid="{4CD09CAB-0916-4781-8563-ED2858AE636F}" name="Is_Beginning_Number"/>
   </tableColumns>
@@ -3066,34 +3117,34 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADB8C96C-1591-5F48-A392-4D1EC7052CD5}" name="Table1" displayName="Table1" ref="B1:V11" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADB8C96C-1591-5F48-A392-4D1EC7052CD5}" name="Table1" displayName="Table1" ref="B1:V11" totalsRowShown="0" headerRowDxfId="24" dataDxfId="23">
   <autoFilter ref="B1:V11" xr:uid="{ADB8C96C-1591-5F48-A392-4D1EC7052CD5}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{E978C108-A1D4-384A-A65D-5CDA04CE21F8}" name="OBJECTIVE " dataDxfId="20"/>
-    <tableColumn id="2" xr3:uid="{52FB3C8C-5116-474B-B994-EED1FE49CD47}" name="GOAL " dataDxfId="19"/>
-    <tableColumn id="9" xr3:uid="{938EFC11-14E9-4DC4-9F2A-9A73A924EC9A}" name="How to get data" dataDxfId="18"/>
-    <tableColumn id="3" xr3:uid="{CCA3F28E-50D1-B846-A48A-304C1FBEC00A}" name="Measure/Target" dataDxfId="17"/>
-    <tableColumn id="4" xr3:uid="{9C63CC9A-09B2-E844-8019-0E240D77A6A6}" name="Beginning Number (Nov 2025)" dataDxfId="16"/>
-    <tableColumn id="16" xr3:uid="{5CD65D6C-DF09-453D-BD80-045B5CDB42CF}" name="Sep-25" dataDxfId="15"/>
-    <tableColumn id="15" xr3:uid="{9E58C254-0303-4E66-AA69-5AEC95C512AB}" name="Oct-25" dataDxfId="14"/>
-    <tableColumn id="14" xr3:uid="{17FA72D6-91C0-4EED-A68F-16ACCA76C12C}" name="Nov-25" dataDxfId="13"/>
-    <tableColumn id="13" xr3:uid="{B088E159-7AFB-408F-8F10-9384CBE3394B}" name="Dec-25" dataDxfId="12"/>
-    <tableColumn id="17" xr3:uid="{35DED57A-D3EC-42B0-BAE2-25E758571065}" name="Jan-26" dataDxfId="11"/>
-    <tableColumn id="18" xr3:uid="{49CA4A79-4F20-4E93-9001-FCE8B0B05161}" name="Feb-26" dataDxfId="10"/>
-    <tableColumn id="19" xr3:uid="{11FA3AA1-1AF9-4EEA-AB08-F6BC2A9FA856}" name="Mar-26" dataDxfId="9"/>
-    <tableColumn id="10" xr3:uid="{C616DE4A-6DC6-8446-BF38-C05DEBBEAE05}" name="Apr-26" dataDxfId="8"/>
-    <tableColumn id="12" xr3:uid="{4FE166E4-10BC-754E-97AE-CE2B9C7C4A59}" name="May-26" dataDxfId="7"/>
-    <tableColumn id="11" xr3:uid="{D648C3C7-DBBE-1643-9F59-3BBAF9BE5370}" name="Jun-26" dataDxfId="6"/>
-    <tableColumn id="21" xr3:uid="{B3B9BF37-EA8B-4417-BCDC-B8E1DEB50C36}" name="Jul-26" dataDxfId="5"/>
-    <tableColumn id="20" xr3:uid="{E54D1739-198D-4E98-983F-506C470DEC23}" name="Aug-26" dataDxfId="4"/>
-    <tableColumn id="5" xr3:uid="{DCC50E8E-6C5E-F74F-A300-85E288C1D1CD}" name="Actual/Current" dataDxfId="3"/>
-    <tableColumn id="6" xr3:uid="{DFB92422-1384-034C-A32E-F78EAB900009}" name="% Completed" dataDxfId="2">
+    <tableColumn id="1" xr3:uid="{E978C108-A1D4-384A-A65D-5CDA04CE21F8}" name="OBJECTIVE " dataDxfId="22"/>
+    <tableColumn id="2" xr3:uid="{52FB3C8C-5116-474B-B994-EED1FE49CD47}" name="GOAL " dataDxfId="21"/>
+    <tableColumn id="9" xr3:uid="{938EFC11-14E9-4DC4-9F2A-9A73A924EC9A}" name="How to get data" dataDxfId="20"/>
+    <tableColumn id="3" xr3:uid="{CCA3F28E-50D1-B846-A48A-304C1FBEC00A}" name="Measure/Target" dataDxfId="19"/>
+    <tableColumn id="4" xr3:uid="{9C63CC9A-09B2-E844-8019-0E240D77A6A6}" name="Beginning Number (Nov 2025)" dataDxfId="18"/>
+    <tableColumn id="16" xr3:uid="{5CD65D6C-DF09-453D-BD80-045B5CDB42CF}" name="Sep-25" dataDxfId="17"/>
+    <tableColumn id="15" xr3:uid="{9E58C254-0303-4E66-AA69-5AEC95C512AB}" name="Oct-25" dataDxfId="16"/>
+    <tableColumn id="14" xr3:uid="{17FA72D6-91C0-4EED-A68F-16ACCA76C12C}" name="Nov-25" dataDxfId="15"/>
+    <tableColumn id="13" xr3:uid="{B088E159-7AFB-408F-8F10-9384CBE3394B}" name="Dec-25" dataDxfId="14"/>
+    <tableColumn id="17" xr3:uid="{35DED57A-D3EC-42B0-BAE2-25E758571065}" name="Jan-26" dataDxfId="13"/>
+    <tableColumn id="18" xr3:uid="{49CA4A79-4F20-4E93-9001-FCE8B0B05161}" name="Feb-26" dataDxfId="12"/>
+    <tableColumn id="19" xr3:uid="{11FA3AA1-1AF9-4EEA-AB08-F6BC2A9FA856}" name="Mar-26" dataDxfId="11"/>
+    <tableColumn id="10" xr3:uid="{C616DE4A-6DC6-8446-BF38-C05DEBBEAE05}" name="Apr-26" dataDxfId="10"/>
+    <tableColumn id="12" xr3:uid="{4FE166E4-10BC-754E-97AE-CE2B9C7C4A59}" name="May-26" dataDxfId="9"/>
+    <tableColumn id="11" xr3:uid="{D648C3C7-DBBE-1643-9F59-3BBAF9BE5370}" name="Jun-26" dataDxfId="8"/>
+    <tableColumn id="21" xr3:uid="{B3B9BF37-EA8B-4417-BCDC-B8E1DEB50C36}" name="Jul-26" dataDxfId="7"/>
+    <tableColumn id="20" xr3:uid="{E54D1739-198D-4E98-983F-506C470DEC23}" name="Aug-26" dataDxfId="6"/>
+    <tableColumn id="5" xr3:uid="{DCC50E8E-6C5E-F74F-A300-85E288C1D1CD}" name="Actual/Current" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{DFB92422-1384-034C-A32E-F78EAB900009}" name="% Completed" dataDxfId="4">
       <calculatedColumnFormula>IFERROR(S2/F2,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{291AF90F-1804-3448-9A9C-A334F495B9CD}" name="Left to do" dataDxfId="1">
+    <tableColumn id="7" xr3:uid="{291AF90F-1804-3448-9A9C-A334F495B9CD}" name="Left to do" dataDxfId="3">
       <calculatedColumnFormula>F2-S2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{77A9B761-776A-334E-9110-B7F7E9CA082B}" name="Notes" dataDxfId="0"/>
+    <tableColumn id="8" xr3:uid="{77A9B761-776A-334E-9110-B7F7E9CA082B}" name="Notes" dataDxfId="2"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5518,26 +5569,26 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
-      <c r="A1" t="s">
+      <c r="A1" s="99" t="s">
         <v>240</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="99" t="s">
         <v>241</v>
       </c>
     </row>
     <row r="2" spans="1:2">
-      <c r="A2">
+      <c r="A2" s="98">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="98" t="s">
         <v>242</v>
       </c>
     </row>
     <row r="3" spans="1:2">
-      <c r="A3">
+      <c r="A3" s="100">
         <v>2</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B3" s="100" t="s">
         <v>243</v>
       </c>
     </row>
@@ -7597,15 +7648,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010067C3E934A0AA0B40A01BB34EE44DBE4E" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="99f90e1838b691a269ec0be7c9d3b1c4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7bc4fa38-d888-4f67-9acc-d35155363a39" xmlns:ns3="fff59cbe-7145-45c6-b0b8-a33a9ec94a75" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="55b527a863acd720578db25cd4da17b2" ns2:_="" ns3:_="">
     <xsd:import namespace="7bc4fa38-d888-4f67-9acc-d35155363a39"/>
@@ -7800,6 +7842,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9F09B98-3A3F-4A19-9439-839483AD047D}">
   <ds:schemaRefs>
@@ -7818,14 +7869,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57AD8670-20BC-4534-A7A5-87984349E00F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{339BB920-340D-4757-A55F-4B7C981C835F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -7842,4 +7885,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57AD8670-20BC-4534-A7A5-87984349E00F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
fix(dax): update [Actual_Status] to ignore pre-populated zeroes
Modified the MAX date evaluation to filter for 'Actual_Value <> 0' instead of NOT ISBLANK. This correctly identifies the latest actual progression value, bypassing future months that default to zero in the 'results' table.
</commit_message>
<xml_diff>
--- a/Datasets/okrs.xlsx
+++ b/Datasets/okrs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauro\Desktop\Accenture\Dashboard okrs\Datasets\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauro.turner\Proyectos\Dashboards\Global-IT---OKR-KPI-Dashboard\Datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78B2621F-BFDE-45BD-B7B4-21AC2916F99F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0D0F15-C948-4C6A-8A14-6A59F7FA4593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" tabRatio="810" activeTab="7" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="810" activeTab="7" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
   </bookViews>
   <sheets>
     <sheet name="objetives" sheetId="11" r:id="rId1"/>
@@ -58,17 +58,17 @@
   <commentList>
     <comment ref="M2" authorId="0" shapeId="0" xr:uid="{DB759141-B278-42B0-A911-47F9208B482B}">
       <text>
-        <t>[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Big change due to change in filters</t>
       </text>
     </comment>
     <comment ref="L3" authorId="1" shapeId="0" xr:uid="{01E69275-C16E-4D70-A498-1B10AE23770E}">
       <text>
-        <t>[Comentario encadenado]
-Su versión de Excel le permite leer este comentario encadenado; sin embargo, las ediciones que se apliquen se quitarán si el archivo se abre en una versión más reciente de Excel. Más información: https://go.microsoft.com/fwlink/?linkid=870924
-Comentario:
+        <t>[Threaded comment]
+Your version of Excel allows you to read this threaded comment; however, any edits to it will get removed if the file is opened in a newer version of Excel. Learn more: https://go.microsoft.com/fwlink/?linkid=870924
+Comment:
     Q2 (as-of 3/4): 87.27%
 Not Q2 snapshot yet</t>
       </text>
@@ -1297,8 +1297,8 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="2">
-    <numFmt numFmtId="169" formatCode="m/d/yy;@"/>
-    <numFmt numFmtId="170" formatCode="[$-1540A]m/d/yyyy;@"/>
+    <numFmt numFmtId="164" formatCode="m/d/yy;@"/>
+    <numFmt numFmtId="165" formatCode="[$-1540A]m/d/yyyy;@"/>
   </numFmts>
   <fonts count="32">
     <font>
@@ -1718,7 +1718,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="104">
+  <cellXfs count="103">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1986,18 +1986,14 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
-    <xf numFmtId="169" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="170" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
-    <cellStyle name="Porcentaje" xfId="1" builtinId="5"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="26">
-    <dxf>
-      <numFmt numFmtId="170" formatCode="[$-1540A]m/d/yyyy;@"/>
-    </dxf>
     <dxf>
       <font>
         <strike val="0"/>
@@ -2377,6 +2373,9 @@
         </patternFill>
       </fill>
       <alignment horizontal="center" vertical="center" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="[$-1540A]m/d/yyyy;@"/>
     </dxf>
     <dxf>
       <border outline="0">
@@ -3115,7 +3114,7 @@
   <tableColumns count="5">
     <tableColumn id="1" xr3:uid="{D2F6C869-298A-4690-A078-35A0D201E072}" name="Result_ID"/>
     <tableColumn id="2" xr3:uid="{3F7B7E26-AE5E-4B25-BEF0-6F64A9729CC1}" name="KPI_ID"/>
-    <tableColumn id="3" xr3:uid="{1AEA6639-430E-4250-A1EC-1DCF4FC5151B}" name="Date" dataDxfId="0"/>
+    <tableColumn id="3" xr3:uid="{1AEA6639-430E-4250-A1EC-1DCF4FC5151B}" name="Date" dataDxfId="23"/>
     <tableColumn id="4" xr3:uid="{96F10FB5-5453-4273-8C7D-2EB9CF434694}" name="Actual_Value"/>
     <tableColumn id="5" xr3:uid="{4CD09CAB-0916-4781-8563-ED2858AE636F}" name="Is_Beginning_Number"/>
   </tableColumns>
@@ -3124,34 +3123,34 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADB8C96C-1591-5F48-A392-4D1EC7052CD5}" name="Table1" displayName="Table1" ref="B1:V11" totalsRowShown="0" headerRowDxfId="23" dataDxfId="22">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADB8C96C-1591-5F48-A392-4D1EC7052CD5}" name="Table1" displayName="Table1" ref="B1:V11" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="B1:V11" xr:uid="{ADB8C96C-1591-5F48-A392-4D1EC7052CD5}"/>
   <tableColumns count="21">
-    <tableColumn id="1" xr3:uid="{E978C108-A1D4-384A-A65D-5CDA04CE21F8}" name="OBJECTIVE " dataDxfId="21"/>
-    <tableColumn id="2" xr3:uid="{52FB3C8C-5116-474B-B994-EED1FE49CD47}" name="GOAL " dataDxfId="20"/>
-    <tableColumn id="9" xr3:uid="{938EFC11-14E9-4DC4-9F2A-9A73A924EC9A}" name="How to get data" dataDxfId="19"/>
-    <tableColumn id="3" xr3:uid="{CCA3F28E-50D1-B846-A48A-304C1FBEC00A}" name="Measure/Target" dataDxfId="18"/>
-    <tableColumn id="4" xr3:uid="{9C63CC9A-09B2-E844-8019-0E240D77A6A6}" name="Beginning Number (Nov 2025)" dataDxfId="17"/>
-    <tableColumn id="16" xr3:uid="{5CD65D6C-DF09-453D-BD80-045B5CDB42CF}" name="sep-25" dataDxfId="16"/>
-    <tableColumn id="15" xr3:uid="{9E58C254-0303-4E66-AA69-5AEC95C512AB}" name="Oct-25" dataDxfId="15"/>
-    <tableColumn id="14" xr3:uid="{17FA72D6-91C0-4EED-A68F-16ACCA76C12C}" name="Nov-25" dataDxfId="14"/>
-    <tableColumn id="13" xr3:uid="{B088E159-7AFB-408F-8F10-9384CBE3394B}" name="Dec-25" dataDxfId="13"/>
-    <tableColumn id="17" xr3:uid="{35DED57A-D3EC-42B0-BAE2-25E758571065}" name="Jan-26" dataDxfId="12"/>
-    <tableColumn id="18" xr3:uid="{49CA4A79-4F20-4E93-9001-FCE8B0B05161}" name="Feb-26" dataDxfId="11"/>
-    <tableColumn id="19" xr3:uid="{11FA3AA1-1AF9-4EEA-AB08-F6BC2A9FA856}" name="Mar-26" dataDxfId="10"/>
-    <tableColumn id="10" xr3:uid="{C616DE4A-6DC6-8446-BF38-C05DEBBEAE05}" name="Apr-26" dataDxfId="9"/>
-    <tableColumn id="12" xr3:uid="{4FE166E4-10BC-754E-97AE-CE2B9C7C4A59}" name="May-26" dataDxfId="8"/>
-    <tableColumn id="11" xr3:uid="{D648C3C7-DBBE-1643-9F59-3BBAF9BE5370}" name="Jun-26" dataDxfId="7"/>
-    <tableColumn id="21" xr3:uid="{B3B9BF37-EA8B-4417-BCDC-B8E1DEB50C36}" name="Jul-26" dataDxfId="6"/>
-    <tableColumn id="20" xr3:uid="{E54D1739-198D-4E98-983F-506C470DEC23}" name="Aug-26" dataDxfId="5"/>
-    <tableColumn id="5" xr3:uid="{DCC50E8E-6C5E-F74F-A300-85E288C1D1CD}" name="Actual/Current" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{DFB92422-1384-034C-A32E-F78EAB900009}" name="% Completed" dataDxfId="3">
+    <tableColumn id="1" xr3:uid="{E978C108-A1D4-384A-A65D-5CDA04CE21F8}" name="OBJECTIVE " dataDxfId="20"/>
+    <tableColumn id="2" xr3:uid="{52FB3C8C-5116-474B-B994-EED1FE49CD47}" name="GOAL " dataDxfId="19"/>
+    <tableColumn id="9" xr3:uid="{938EFC11-14E9-4DC4-9F2A-9A73A924EC9A}" name="How to get data" dataDxfId="18"/>
+    <tableColumn id="3" xr3:uid="{CCA3F28E-50D1-B846-A48A-304C1FBEC00A}" name="Measure/Target" dataDxfId="17"/>
+    <tableColumn id="4" xr3:uid="{9C63CC9A-09B2-E844-8019-0E240D77A6A6}" name="Beginning Number (Nov 2025)" dataDxfId="16"/>
+    <tableColumn id="16" xr3:uid="{5CD65D6C-DF09-453D-BD80-045B5CDB42CF}" name="sep-25" dataDxfId="15"/>
+    <tableColumn id="15" xr3:uid="{9E58C254-0303-4E66-AA69-5AEC95C512AB}" name="Oct-25" dataDxfId="14"/>
+    <tableColumn id="14" xr3:uid="{17FA72D6-91C0-4EED-A68F-16ACCA76C12C}" name="Nov-25" dataDxfId="13"/>
+    <tableColumn id="13" xr3:uid="{B088E159-7AFB-408F-8F10-9384CBE3394B}" name="Dec-25" dataDxfId="12"/>
+    <tableColumn id="17" xr3:uid="{35DED57A-D3EC-42B0-BAE2-25E758571065}" name="Jan-26" dataDxfId="11"/>
+    <tableColumn id="18" xr3:uid="{49CA4A79-4F20-4E93-9001-FCE8B0B05161}" name="Feb-26" dataDxfId="10"/>
+    <tableColumn id="19" xr3:uid="{11FA3AA1-1AF9-4EEA-AB08-F6BC2A9FA856}" name="Mar-26" dataDxfId="9"/>
+    <tableColumn id="10" xr3:uid="{C616DE4A-6DC6-8446-BF38-C05DEBBEAE05}" name="Apr-26" dataDxfId="8"/>
+    <tableColumn id="12" xr3:uid="{4FE166E4-10BC-754E-97AE-CE2B9C7C4A59}" name="May-26" dataDxfId="7"/>
+    <tableColumn id="11" xr3:uid="{D648C3C7-DBBE-1643-9F59-3BBAF9BE5370}" name="Jun-26" dataDxfId="6"/>
+    <tableColumn id="21" xr3:uid="{B3B9BF37-EA8B-4417-BCDC-B8E1DEB50C36}" name="Jul-26" dataDxfId="5"/>
+    <tableColumn id="20" xr3:uid="{E54D1739-198D-4E98-983F-506C470DEC23}" name="Aug-26" dataDxfId="4"/>
+    <tableColumn id="5" xr3:uid="{DCC50E8E-6C5E-F74F-A300-85E288C1D1CD}" name="Actual/Current" dataDxfId="3"/>
+    <tableColumn id="6" xr3:uid="{DFB92422-1384-034C-A32E-F78EAB900009}" name="% Completed" dataDxfId="2">
       <calculatedColumnFormula>IFERROR(S2/F2,0)</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="7" xr3:uid="{291AF90F-1804-3448-9A9C-A334F495B9CD}" name="Left to do" dataDxfId="2">
+    <tableColumn id="7" xr3:uid="{291AF90F-1804-3448-9A9C-A334F495B9CD}" name="Left to do" dataDxfId="1">
       <calculatedColumnFormula>F2-S2</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="8" xr3:uid="{77A9B761-776A-334E-9110-B7F7E9CA082B}" name="Notes" dataDxfId="1"/>
+    <tableColumn id="8" xr3:uid="{77A9B761-776A-334E-9110-B7F7E9CA082B}" name="Notes" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -3487,7 +3486,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{813D2C94-41CC-4AE7-B170-6BA14640E37E}">
   <dimension ref="A1:B4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="12" customWidth="1"/>
   </cols>
@@ -3535,7 +3534,7 @@
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A1C2DE-958E-4EF5-BD32-D7572A596892}">
   <dimension ref="A1:C81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" s="57">
@@ -3617,11 +3616,11 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A5511CF-ECA4-4801-B421-12A212CAD755}">
   <dimension ref="A1:R81"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="17.125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="17.08203125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="25.625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="25.58203125" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="31" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -3658,7 +3657,7 @@
         <v>63</v>
       </c>
     </row>
-    <row r="15" spans="1:18" ht="110.25">
+    <row r="15" spans="1:18" ht="112">
       <c r="D15" t="s">
         <v>180</v>
       </c>
@@ -3885,7 +3884,7 @@
         <v>183</v>
       </c>
     </row>
-    <row r="53" spans="1:4" ht="47.25">
+    <row r="53" spans="1:4" ht="48">
       <c r="A53" s="85" t="s">
         <v>184</v>
       </c>
@@ -3899,7 +3898,7 @@
         <v>0.83109999999999995</v>
       </c>
     </row>
-    <row r="54" spans="1:4" ht="63">
+    <row r="54" spans="1:4" ht="64">
       <c r="A54" s="85" t="s">
         <v>185</v>
       </c>
@@ -3913,7 +3912,7 @@
         <v>0.83340000000000003</v>
       </c>
     </row>
-    <row r="55" spans="1:4" ht="63">
+    <row r="55" spans="1:4" ht="64">
       <c r="A55" s="85" t="s">
         <v>186</v>
       </c>
@@ -3927,7 +3926,7 @@
         <v>0.85740000000000005</v>
       </c>
     </row>
-    <row r="56" spans="1:4" ht="63">
+    <row r="56" spans="1:4" ht="64">
       <c r="A56" s="85" t="s">
         <v>187</v>
       </c>
@@ -3941,7 +3940,7 @@
         <v>0.86839999999999995</v>
       </c>
     </row>
-    <row r="57" spans="1:4" ht="63">
+    <row r="57" spans="1:4" ht="64">
       <c r="A57" s="85" t="s">
         <v>188</v>
       </c>
@@ -3955,7 +3954,7 @@
         <v>0.87009999999999998</v>
       </c>
     </row>
-    <row r="58" spans="1:4" ht="63">
+    <row r="58" spans="1:4" ht="64">
       <c r="A58" s="85" t="s">
         <v>189</v>
       </c>
@@ -3969,7 +3968,7 @@
         <v>0.87180000000000002</v>
       </c>
     </row>
-    <row r="59" spans="1:4" ht="47.25">
+    <row r="59" spans="1:4" ht="48">
       <c r="A59" s="85" t="s">
         <v>190</v>
       </c>
@@ -3983,7 +3982,7 @@
         <v>0.87390000000000001</v>
       </c>
     </row>
-    <row r="60" spans="1:4" ht="47.25">
+    <row r="60" spans="1:4" ht="48">
       <c r="A60" s="85" t="s">
         <v>191</v>
       </c>
@@ -3997,7 +3996,7 @@
         <v>0.87939999999999996</v>
       </c>
     </row>
-    <row r="61" spans="1:4" ht="47.25">
+    <row r="61" spans="1:4" ht="48">
       <c r="A61" s="85" t="s">
         <v>192</v>
       </c>
@@ -4011,7 +4010,7 @@
         <v>0.88719999999999999</v>
       </c>
     </row>
-    <row r="62" spans="1:4" ht="47.25">
+    <row r="62" spans="1:4" ht="48">
       <c r="A62" s="85" t="s">
         <v>193</v>
       </c>
@@ -4025,7 +4024,7 @@
         <v>0.89219999999999999</v>
       </c>
     </row>
-    <row r="63" spans="1:4" ht="47.25">
+    <row r="63" spans="1:4" ht="48">
       <c r="A63" s="85" t="s">
         <v>194</v>
       </c>
@@ -4039,7 +4038,7 @@
         <v>0.89339999999999997</v>
       </c>
     </row>
-    <row r="64" spans="1:4" ht="47.25">
+    <row r="64" spans="1:4" ht="48">
       <c r="A64" s="85" t="s">
         <v>195</v>
       </c>
@@ -4053,7 +4052,7 @@
         <v>0.9012</v>
       </c>
     </row>
-    <row r="65" spans="1:4" ht="47.25">
+    <row r="65" spans="1:4" ht="48">
       <c r="A65" s="85" t="s">
         <v>196</v>
       </c>
@@ -4067,7 +4066,7 @@
         <v>0.90659999999999996</v>
       </c>
     </row>
-    <row r="66" spans="1:4" ht="47.25">
+    <row r="66" spans="1:4" ht="48">
       <c r="A66" s="85" t="s">
         <v>197</v>
       </c>
@@ -4150,10 +4149,10 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BAD0912-E0CB-460C-ABF0-F667933348DC}">
   <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
     <col min="1" max="1" width="26.5" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="41.375" customWidth="1"/>
+    <col min="2" max="2" width="41.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -4180,7 +4179,7 @@
         <v>46366</v>
       </c>
     </row>
-    <row r="4" spans="1:2" ht="31.5">
+    <row r="4" spans="1:2" ht="32">
       <c r="A4" s="39" t="s">
         <v>40</v>
       </c>
@@ -4188,7 +4187,7 @@
         <v>46050</v>
       </c>
     </row>
-    <row r="5" spans="1:2" ht="31.5">
+    <row r="5" spans="1:2" ht="32">
       <c r="A5" s="39" t="s">
         <v>41</v>
       </c>
@@ -4212,13 +4211,13 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FECA49D2-6EDF-4BD1-9DAB-FC593DCBD3BD}">
   <dimension ref="A2:H78"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
   <cols>
-    <col min="1" max="1" width="14.625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="18.375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.58203125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.33203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="56.5" customWidth="1"/>
-    <col min="4" max="4" width="41.875" customWidth="1"/>
-    <col min="6" max="6" width="22.375" customWidth="1"/>
+    <col min="4" max="4" width="41.83203125" customWidth="1"/>
+    <col min="6" max="6" width="22.33203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="2" spans="8:8">
@@ -4719,7 +4718,7 @@
         <v>112</v>
       </c>
     </row>
-    <row r="51" spans="1:6" s="72" customFormat="1" ht="13.5">
+    <row r="51" spans="1:6" s="72" customFormat="1" ht="13">
       <c r="A51" s="68" t="s">
         <v>113</v>
       </c>
@@ -4739,7 +4738,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="52" spans="1:6" s="72" customFormat="1" ht="67.5">
+    <row r="52" spans="1:6" s="72" customFormat="1" ht="65">
       <c r="A52" s="73" t="s">
         <v>119</v>
       </c>
@@ -4759,7 +4758,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="53" spans="1:6" s="72" customFormat="1" ht="67.5">
+    <row r="53" spans="1:6" s="72" customFormat="1" ht="65">
       <c r="A53" s="79" t="s">
         <v>119</v>
       </c>
@@ -4779,7 +4778,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="54" spans="1:6" s="72" customFormat="1" ht="135">
+    <row r="54" spans="1:6" s="72" customFormat="1" ht="130">
       <c r="A54" s="73" t="s">
         <v>119</v>
       </c>
@@ -4799,7 +4798,7 @@
         <v>128</v>
       </c>
     </row>
-    <row r="55" spans="1:6" s="72" customFormat="1" ht="121.5">
+    <row r="55" spans="1:6" s="72" customFormat="1" ht="117">
       <c r="A55" s="79" t="s">
         <v>119</v>
       </c>
@@ -4819,7 +4818,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="56" spans="1:6" s="72" customFormat="1" ht="108">
+    <row r="56" spans="1:6" s="72" customFormat="1" ht="104">
       <c r="A56" s="73" t="s">
         <v>119</v>
       </c>
@@ -4839,7 +4838,7 @@
         <v>132</v>
       </c>
     </row>
-    <row r="57" spans="1:6" s="72" customFormat="1" ht="67.5">
+    <row r="57" spans="1:6" s="72" customFormat="1" ht="65">
       <c r="A57" s="79" t="s">
         <v>119</v>
       </c>
@@ -4859,7 +4858,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="58" spans="1:6" s="72" customFormat="1" ht="135">
+    <row r="58" spans="1:6" s="72" customFormat="1" ht="130">
       <c r="A58" s="73" t="s">
         <v>119</v>
       </c>
@@ -4879,7 +4878,7 @@
         <v>137</v>
       </c>
     </row>
-    <row r="59" spans="1:6" s="72" customFormat="1" ht="162">
+    <row r="59" spans="1:6" s="72" customFormat="1" ht="156">
       <c r="A59" s="79" t="s">
         <v>119</v>
       </c>
@@ -4899,7 +4898,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="60" spans="1:6" s="72" customFormat="1" ht="94.5">
+    <row r="60" spans="1:6" s="72" customFormat="1" ht="91">
       <c r="A60" s="73" t="s">
         <v>119</v>
       </c>
@@ -4919,7 +4918,7 @@
         <v>142</v>
       </c>
     </row>
-    <row r="61" spans="1:6" s="72" customFormat="1" ht="189">
+    <row r="61" spans="1:6" s="72" customFormat="1" ht="182">
       <c r="A61" s="79" t="s">
         <v>119</v>
       </c>
@@ -4939,7 +4938,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="62" spans="1:6" s="72" customFormat="1" ht="162">
+    <row r="62" spans="1:6" s="72" customFormat="1" ht="156">
       <c r="A62" s="73" t="s">
         <v>119</v>
       </c>
@@ -4959,7 +4958,7 @@
         <v>146</v>
       </c>
     </row>
-    <row r="63" spans="1:6" s="72" customFormat="1" ht="229.5">
+    <row r="63" spans="1:6" s="72" customFormat="1" ht="221">
       <c r="A63" s="79" t="s">
         <v>119</v>
       </c>
@@ -4979,7 +4978,7 @@
         <v>148</v>
       </c>
     </row>
-    <row r="64" spans="1:6" s="72" customFormat="1" ht="270">
+    <row r="64" spans="1:6" s="72" customFormat="1" ht="260">
       <c r="A64" s="73" t="s">
         <v>119</v>
       </c>
@@ -5019,7 +5018,7 @@
         <v>152</v>
       </c>
     </row>
-    <row r="66" spans="1:6" s="72" customFormat="1" ht="351">
+    <row r="66" spans="1:6" s="72" customFormat="1" ht="338">
       <c r="A66" s="73" t="s">
         <v>119</v>
       </c>
@@ -5039,7 +5038,7 @@
         <v>154</v>
       </c>
     </row>
-    <row r="67" spans="1:6" s="72" customFormat="1" ht="270">
+    <row r="67" spans="1:6" s="72" customFormat="1" ht="273">
       <c r="A67" s="79" t="s">
         <v>119</v>
       </c>
@@ -5059,7 +5058,7 @@
         <v>156</v>
       </c>
     </row>
-    <row r="68" spans="1:6" s="72" customFormat="1" ht="108">
+    <row r="68" spans="1:6" s="72" customFormat="1" ht="104">
       <c r="A68" s="73" t="s">
         <v>119</v>
       </c>
@@ -5079,7 +5078,7 @@
         <v>158</v>
       </c>
     </row>
-    <row r="69" spans="1:6" s="72" customFormat="1" ht="67.5">
+    <row r="69" spans="1:6" s="72" customFormat="1" ht="65">
       <c r="A69" s="79" t="s">
         <v>119</v>
       </c>
@@ -5099,7 +5098,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="70" spans="1:6" s="72" customFormat="1" ht="54">
+    <row r="70" spans="1:6" s="72" customFormat="1" ht="52">
       <c r="A70" s="73" t="s">
         <v>119</v>
       </c>
@@ -5119,7 +5118,7 @@
         <v>162</v>
       </c>
     </row>
-    <row r="71" spans="1:6" s="72" customFormat="1" ht="54">
+    <row r="71" spans="1:6" s="72" customFormat="1" ht="52">
       <c r="A71" s="79" t="s">
         <v>119</v>
       </c>
@@ -5139,7 +5138,7 @@
         <v>164</v>
       </c>
     </row>
-    <row r="72" spans="1:6" s="72" customFormat="1" ht="67.5">
+    <row r="72" spans="1:6" s="72" customFormat="1" ht="65">
       <c r="A72" s="73" t="s">
         <v>119</v>
       </c>
@@ -5159,7 +5158,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="73" spans="1:6" s="72" customFormat="1" ht="54">
+    <row r="73" spans="1:6" s="72" customFormat="1" ht="52">
       <c r="A73" s="79" t="s">
         <v>119</v>
       </c>
@@ -5179,7 +5178,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="74" spans="1:6" s="72" customFormat="1" ht="27">
+    <row r="74" spans="1:6" s="72" customFormat="1" ht="26">
       <c r="A74" s="73" t="s">
         <v>119</v>
       </c>
@@ -5199,7 +5198,7 @@
         <v>170</v>
       </c>
     </row>
-    <row r="75" spans="1:6" s="72" customFormat="1" ht="54">
+    <row r="75" spans="1:6" s="72" customFormat="1" ht="52">
       <c r="A75" s="79" t="s">
         <v>119</v>
       </c>
@@ -5219,7 +5218,7 @@
         <v>172</v>
       </c>
     </row>
-    <row r="76" spans="1:6" s="72" customFormat="1" ht="67.5">
+    <row r="76" spans="1:6" s="72" customFormat="1" ht="65">
       <c r="A76" s="73" t="s">
         <v>119</v>
       </c>
@@ -5239,7 +5238,7 @@
         <v>174</v>
       </c>
     </row>
-    <row r="77" spans="1:6" s="72" customFormat="1" ht="162">
+    <row r="77" spans="1:6" s="72" customFormat="1" ht="156">
       <c r="A77" s="79" t="s">
         <v>119</v>
       </c>
@@ -5259,7 +5258,7 @@
         <v>176</v>
       </c>
     </row>
-    <row r="78" spans="1:6" s="72" customFormat="1" ht="94.5">
+    <row r="78" spans="1:6" s="72" customFormat="1" ht="91">
       <c r="A78" s="73" t="s">
         <v>119</v>
       </c>
@@ -5288,54 +5287,54 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92D61564-BD00-449F-B779-9A392A403D13}">
   <dimension ref="A2:A14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
   <sheetData>
-    <row r="2" spans="1:1" ht="18.75">
+    <row r="2" spans="1:1" ht="21.5">
       <c r="A2" s="53" t="s">
         <v>52</v>
       </c>
     </row>
-    <row r="3" spans="1:1" ht="18">
+    <row r="3" spans="1:1" ht="21.5">
       <c r="A3" s="52" t="s">
         <v>53</v>
       </c>
     </row>
-    <row r="4" spans="1:1" ht="18">
+    <row r="4" spans="1:1" ht="21.5">
       <c r="A4" s="52" t="s">
         <v>54</v>
       </c>
     </row>
-    <row r="5" spans="1:1" ht="18">
+    <row r="5" spans="1:1" ht="21.5">
       <c r="A5" s="52" t="s">
         <v>55</v>
       </c>
     </row>
-    <row r="6" spans="1:1" ht="18">
+    <row r="6" spans="1:1" ht="21.5">
       <c r="A6" s="52" t="s">
         <v>56</v>
       </c>
     </row>
-    <row r="8" spans="1:1">
+    <row r="8" spans="1:1" ht="18.5">
       <c r="A8" s="56" t="s">
         <v>57</v>
       </c>
     </row>
-    <row r="9" spans="1:1">
+    <row r="9" spans="1:1" ht="18.5">
       <c r="A9" s="54" t="s">
         <v>58</v>
       </c>
     </row>
-    <row r="10" spans="1:1">
+    <row r="10" spans="1:1" ht="18.5">
       <c r="A10" s="54" t="s">
         <v>59</v>
       </c>
     </row>
-    <row r="11" spans="1:1">
+    <row r="11" spans="1:1" ht="18.5">
       <c r="A11" s="55" t="s">
         <v>60</v>
       </c>
     </row>
-    <row r="12" spans="1:1">
+    <row r="12" spans="1:1" ht="18.5">
       <c r="A12" s="54" t="s">
         <v>61</v>
       </c>
@@ -5353,7 +5352,7 @@
 <file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B73C4F58-E1C8-4D89-93FA-19463BA41BD4}">
   <dimension ref="A1:A3"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:1">
       <c r="A1" t="s">
@@ -5378,7 +5377,7 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{836B3F50-B765-407E-9FD9-76CC32131808}">
   <dimension ref="A1:B9"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="13.75" customWidth="1"/>
   </cols>
@@ -5466,9 +5465,9 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{88FDE7CB-204B-4F0D-95B4-22E4C775FEC9}">
   <dimension ref="A1:B11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
-    <col min="2" max="2" width="14.125" customWidth="1"/>
+    <col min="2" max="2" width="14.08203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:2">
@@ -5570,7 +5569,7 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78397758-3182-4D2B-AEC2-12D8A685B44A}">
   <dimension ref="A1:B3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="2" width="11.75" customWidth="1"/>
   </cols>
@@ -5610,11 +5609,11 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5716ADCC-E36E-44A5-AF6D-43063C282787}">
   <dimension ref="A1:E11"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
-    <col min="2" max="2" width="12.125" customWidth="1"/>
+    <col min="2" max="2" width="12.08203125" customWidth="1"/>
     <col min="4" max="4" width="29.5" customWidth="1"/>
-    <col min="5" max="5" width="13.125" customWidth="1"/>
+    <col min="5" max="5" width="13.08203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5">
@@ -5809,7 +5808,7 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3992BCCC-153D-40F1-88B0-57A653F9FE93}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -5942,7 +5941,7 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6411490B-BC0C-412A-8052-05A3565BEF25}">
   <dimension ref="A1:B15"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" t="s">
@@ -6075,9 +6074,9 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E88F946-79CD-4577-8C70-9BE607ED0BF5}">
   <dimension ref="A1:Q124"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
-    <col min="4" max="4" width="13.375" customWidth="1"/>
+    <col min="4" max="4" width="13.33203125" customWidth="1"/>
     <col min="5" max="5" width="20" customWidth="1"/>
   </cols>
   <sheetData>
@@ -6114,7 +6113,6 @@
       <c r="E2" t="s">
         <v>248</v>
       </c>
-      <c r="G2" s="103"/>
       <c r="J2" s="101"/>
     </row>
     <row r="3" spans="1:10">
@@ -6133,7 +6131,6 @@
       <c r="E3" t="s">
         <v>248</v>
       </c>
-      <c r="G3" s="103"/>
       <c r="J3" s="101"/>
     </row>
     <row r="4" spans="1:10">
@@ -6147,12 +6144,11 @@
         <v>45962</v>
       </c>
       <c r="D4">
-        <v>986</v>
+        <v>3758</v>
       </c>
       <c r="E4" t="s">
         <v>247</v>
       </c>
-      <c r="G4" s="103"/>
       <c r="J4" s="101"/>
     </row>
     <row r="5" spans="1:10">
@@ -6171,7 +6167,6 @@
       <c r="E5" t="s">
         <v>248</v>
       </c>
-      <c r="G5" s="103"/>
       <c r="J5" s="101"/>
     </row>
     <row r="6" spans="1:10">
@@ -6190,7 +6185,6 @@
       <c r="E6" t="s">
         <v>248</v>
       </c>
-      <c r="G6" s="103"/>
       <c r="J6" s="101"/>
     </row>
     <row r="7" spans="1:10">
@@ -6209,7 +6203,6 @@
       <c r="E7" t="s">
         <v>248</v>
       </c>
-      <c r="G7" s="103"/>
       <c r="J7" s="101"/>
     </row>
     <row r="8" spans="1:10">
@@ -6228,7 +6221,6 @@
       <c r="E8" t="s">
         <v>248</v>
       </c>
-      <c r="G8" s="103"/>
       <c r="J8" s="101"/>
     </row>
     <row r="9" spans="1:10">
@@ -6247,7 +6239,6 @@
       <c r="E9" t="s">
         <v>248</v>
       </c>
-      <c r="G9" s="103"/>
       <c r="J9" s="101"/>
     </row>
     <row r="10" spans="1:10">
@@ -6266,7 +6257,6 @@
       <c r="E10" t="s">
         <v>248</v>
       </c>
-      <c r="G10" s="103"/>
       <c r="J10" s="101"/>
     </row>
     <row r="11" spans="1:10">
@@ -6285,7 +6275,6 @@
       <c r="E11" t="s">
         <v>248</v>
       </c>
-      <c r="G11" s="103"/>
       <c r="J11" s="101"/>
     </row>
     <row r="12" spans="1:10">
@@ -6304,7 +6293,6 @@
       <c r="E12" t="s">
         <v>248</v>
       </c>
-      <c r="G12" s="103"/>
       <c r="J12" s="101"/>
     </row>
     <row r="13" spans="1:10">
@@ -6323,7 +6311,6 @@
       <c r="E13" t="s">
         <v>248</v>
       </c>
-      <c r="G13" s="103"/>
       <c r="J13" s="101"/>
     </row>
     <row r="14" spans="1:10">
@@ -6360,7 +6347,6 @@
       <c r="E15" t="s">
         <v>248</v>
       </c>
-      <c r="G15" s="103"/>
       <c r="J15" s="101"/>
     </row>
     <row r="16" spans="1:10">
@@ -6379,7 +6365,6 @@
       <c r="E16" t="s">
         <v>247</v>
       </c>
-      <c r="G16" s="103"/>
       <c r="J16" s="101"/>
     </row>
     <row r="17" spans="1:15">
@@ -6398,7 +6383,6 @@
       <c r="E17" t="s">
         <v>248</v>
       </c>
-      <c r="G17" s="103"/>
       <c r="J17" s="101"/>
     </row>
     <row r="18" spans="1:15">
@@ -6417,7 +6401,6 @@
       <c r="E18" t="s">
         <v>248</v>
       </c>
-      <c r="G18" s="103"/>
       <c r="J18" s="101"/>
     </row>
     <row r="19" spans="1:15">
@@ -6436,8 +6419,6 @@
       <c r="E19" t="s">
         <v>248</v>
       </c>
-      <c r="G19" s="103"/>
-      <c r="H19" s="103"/>
       <c r="J19" s="101"/>
     </row>
     <row r="20" spans="1:15">
@@ -6456,7 +6437,6 @@
       <c r="E20" t="s">
         <v>248</v>
       </c>
-      <c r="G20" s="103"/>
       <c r="J20" s="101"/>
     </row>
     <row r="21" spans="1:15">
@@ -6475,7 +6455,6 @@
       <c r="E21" t="s">
         <v>248</v>
       </c>
-      <c r="G21" s="103"/>
       <c r="J21" s="101"/>
     </row>
     <row r="22" spans="1:15">
@@ -6494,7 +6473,6 @@
       <c r="E22" t="s">
         <v>248</v>
       </c>
-      <c r="G22" s="103"/>
       <c r="J22" s="101"/>
     </row>
     <row r="23" spans="1:15">
@@ -6513,7 +6491,6 @@
       <c r="E23" t="s">
         <v>248</v>
       </c>
-      <c r="G23" s="103"/>
       <c r="J23" s="101"/>
     </row>
     <row r="24" spans="1:15">
@@ -6532,7 +6509,6 @@
       <c r="E24" t="s">
         <v>248</v>
       </c>
-      <c r="G24" s="103"/>
       <c r="J24" s="101"/>
     </row>
     <row r="25" spans="1:15">
@@ -6551,7 +6527,6 @@
       <c r="E25" t="s">
         <v>248</v>
       </c>
-      <c r="G25" s="103"/>
       <c r="J25" s="101"/>
     </row>
     <row r="26" spans="1:15">
@@ -6570,7 +6545,6 @@
       <c r="E26" t="s">
         <v>248</v>
       </c>
-      <c r="G26" s="103"/>
       <c r="J26" s="101"/>
     </row>
     <row r="27" spans="1:15">
@@ -6589,7 +6563,6 @@
       <c r="E27" t="s">
         <v>248</v>
       </c>
-      <c r="G27" s="103"/>
       <c r="J27" s="101"/>
     </row>
     <row r="28" spans="1:15">
@@ -6608,7 +6581,6 @@
       <c r="E28" t="s">
         <v>247</v>
       </c>
-      <c r="G28" s="103"/>
       <c r="J28" s="101"/>
     </row>
     <row r="29" spans="1:15">
@@ -6627,7 +6599,6 @@
       <c r="E29" t="s">
         <v>248</v>
       </c>
-      <c r="G29" s="103"/>
       <c r="J29" s="101"/>
     </row>
     <row r="30" spans="1:15">
@@ -6646,7 +6617,6 @@
       <c r="E30" t="s">
         <v>248</v>
       </c>
-      <c r="G30" s="103"/>
       <c r="J30" s="101"/>
     </row>
     <row r="31" spans="1:15">
@@ -6665,7 +6635,6 @@
       <c r="E31" t="s">
         <v>248</v>
       </c>
-      <c r="G31" s="103"/>
       <c r="J31" s="101"/>
       <c r="O31" s="57"/>
     </row>
@@ -6685,7 +6654,6 @@
       <c r="E32" t="s">
         <v>248</v>
       </c>
-      <c r="G32" s="103"/>
       <c r="J32" s="101"/>
       <c r="O32" s="57"/>
     </row>
@@ -6705,7 +6673,6 @@
       <c r="E33" t="s">
         <v>248</v>
       </c>
-      <c r="G33" s="103"/>
       <c r="J33" s="101"/>
       <c r="O33" s="57"/>
     </row>
@@ -6725,7 +6692,6 @@
       <c r="E34" t="s">
         <v>248</v>
       </c>
-      <c r="G34" s="103"/>
       <c r="J34" s="101"/>
       <c r="O34" s="57"/>
     </row>
@@ -6745,7 +6711,6 @@
       <c r="E35" t="s">
         <v>248</v>
       </c>
-      <c r="G35" s="103"/>
       <c r="J35" s="101"/>
       <c r="O35" s="57"/>
     </row>
@@ -6765,7 +6730,6 @@
       <c r="E36" t="s">
         <v>248</v>
       </c>
-      <c r="G36" s="103"/>
       <c r="J36" s="101"/>
       <c r="O36" s="57"/>
     </row>
@@ -6785,7 +6749,6 @@
       <c r="E37" t="s">
         <v>248</v>
       </c>
-      <c r="G37" s="103"/>
       <c r="J37" s="101"/>
       <c r="O37" s="57"/>
     </row>
@@ -6805,7 +6768,6 @@
       <c r="E38" t="s">
         <v>248</v>
       </c>
-      <c r="G38" s="103"/>
       <c r="J38" s="101"/>
       <c r="N38" s="57"/>
       <c r="O38" s="57"/>
@@ -6826,7 +6788,6 @@
       <c r="E39" t="s">
         <v>248</v>
       </c>
-      <c r="G39" s="103"/>
       <c r="J39" s="101"/>
       <c r="N39" s="57"/>
       <c r="O39" s="57"/>
@@ -6847,7 +6808,6 @@
       <c r="E40" t="s">
         <v>247</v>
       </c>
-      <c r="G40" s="103"/>
       <c r="J40" s="101"/>
       <c r="N40" s="57"/>
       <c r="O40" s="57"/>
@@ -6868,7 +6828,6 @@
       <c r="E41" t="s">
         <v>248</v>
       </c>
-      <c r="G41" s="103"/>
       <c r="J41" s="101"/>
       <c r="N41" s="57"/>
       <c r="O41" s="57"/>
@@ -6889,7 +6848,6 @@
       <c r="E42" t="s">
         <v>248</v>
       </c>
-      <c r="G42" s="103"/>
       <c r="J42" s="101"/>
       <c r="N42" s="57"/>
       <c r="O42" s="57"/>
@@ -6910,7 +6868,6 @@
       <c r="E43" t="s">
         <v>248</v>
       </c>
-      <c r="G43" s="103"/>
       <c r="J43" s="101"/>
       <c r="N43" s="57"/>
       <c r="O43" s="57"/>
@@ -6931,7 +6888,6 @@
       <c r="E44" t="s">
         <v>248</v>
       </c>
-      <c r="G44" s="103"/>
       <c r="J44" s="101"/>
       <c r="N44" s="57"/>
       <c r="O44" s="57"/>
@@ -6952,7 +6908,6 @@
       <c r="E45" t="s">
         <v>248</v>
       </c>
-      <c r="G45" s="103"/>
       <c r="J45" s="101"/>
       <c r="N45" s="57"/>
       <c r="O45" s="57"/>
@@ -6973,7 +6928,6 @@
       <c r="E46" t="s">
         <v>248</v>
       </c>
-      <c r="G46" s="103"/>
       <c r="J46" s="101"/>
       <c r="N46" s="57"/>
       <c r="O46" s="57"/>
@@ -6994,7 +6948,6 @@
       <c r="E47" t="s">
         <v>248</v>
       </c>
-      <c r="G47" s="103"/>
       <c r="J47" s="101"/>
       <c r="N47" s="57"/>
       <c r="O47" s="57"/>
@@ -7015,7 +6968,6 @@
       <c r="E48" t="s">
         <v>248</v>
       </c>
-      <c r="G48" s="103"/>
       <c r="J48" s="101"/>
       <c r="N48" s="57"/>
       <c r="O48" s="57"/>
@@ -7036,7 +6988,6 @@
       <c r="E49" t="s">
         <v>248</v>
       </c>
-      <c r="G49" s="103"/>
       <c r="J49" s="101"/>
       <c r="L49" s="57"/>
       <c r="N49" s="57"/>
@@ -7058,7 +7009,6 @@
       <c r="E50" t="s">
         <v>248</v>
       </c>
-      <c r="G50" s="103"/>
       <c r="J50" s="101"/>
       <c r="L50" s="57"/>
       <c r="O50" s="57"/>
@@ -7079,7 +7029,6 @@
       <c r="E51" t="s">
         <v>248</v>
       </c>
-      <c r="G51" s="103"/>
       <c r="J51" s="101"/>
       <c r="L51" s="57"/>
       <c r="O51" s="57"/>
@@ -7100,7 +7049,6 @@
       <c r="E52" t="s">
         <v>247</v>
       </c>
-      <c r="G52" s="103"/>
       <c r="J52" s="101"/>
       <c r="L52" s="57"/>
       <c r="O52" s="57"/>
@@ -7121,7 +7069,6 @@
       <c r="E53" t="s">
         <v>248</v>
       </c>
-      <c r="G53" s="103"/>
       <c r="J53" s="101"/>
       <c r="L53" s="57"/>
       <c r="O53" s="57"/>
@@ -7142,7 +7089,6 @@
       <c r="E54" t="s">
         <v>248</v>
       </c>
-      <c r="G54" s="103"/>
       <c r="J54" s="101"/>
       <c r="L54" s="57"/>
     </row>
@@ -7162,7 +7108,6 @@
       <c r="E55" t="s">
         <v>248</v>
       </c>
-      <c r="G55" s="103"/>
       <c r="J55" s="101"/>
       <c r="L55" s="57"/>
     </row>
@@ -7182,7 +7127,6 @@
       <c r="E56" t="s">
         <v>248</v>
       </c>
-      <c r="G56" s="103"/>
       <c r="J56" s="101"/>
       <c r="L56" s="57"/>
     </row>
@@ -7202,7 +7146,6 @@
       <c r="E57" t="s">
         <v>248</v>
       </c>
-      <c r="G57" s="103"/>
       <c r="J57" s="101"/>
       <c r="L57" s="57"/>
     </row>
@@ -7222,7 +7165,6 @@
       <c r="E58" t="s">
         <v>248</v>
       </c>
-      <c r="G58" s="103"/>
       <c r="J58" s="101"/>
       <c r="L58" s="57"/>
     </row>
@@ -7242,7 +7184,6 @@
       <c r="E59" t="s">
         <v>248</v>
       </c>
-      <c r="G59" s="103"/>
       <c r="J59" s="101"/>
       <c r="L59" s="57"/>
     </row>
@@ -7262,7 +7203,6 @@
       <c r="E60" t="s">
         <v>248</v>
       </c>
-      <c r="G60" s="103"/>
       <c r="J60" s="101"/>
       <c r="L60" s="57"/>
     </row>
@@ -7282,7 +7222,6 @@
       <c r="E61" t="s">
         <v>248</v>
       </c>
-      <c r="G61" s="103"/>
       <c r="J61" s="101"/>
     </row>
     <row r="62" spans="1:17">
@@ -7301,7 +7240,6 @@
       <c r="E62" t="s">
         <v>248</v>
       </c>
-      <c r="G62" s="103"/>
       <c r="J62" s="101"/>
     </row>
     <row r="63" spans="1:17">
@@ -7320,7 +7258,6 @@
       <c r="E63" t="s">
         <v>248</v>
       </c>
-      <c r="G63" s="103"/>
       <c r="J63" s="101"/>
       <c r="Q63" s="57"/>
     </row>
@@ -7340,7 +7277,6 @@
       <c r="E64" t="s">
         <v>247</v>
       </c>
-      <c r="G64" s="103"/>
       <c r="J64" s="101"/>
       <c r="Q64" s="57"/>
     </row>
@@ -7360,7 +7296,6 @@
       <c r="E65" t="s">
         <v>248</v>
       </c>
-      <c r="G65" s="103"/>
       <c r="J65" s="101"/>
       <c r="Q65" s="57"/>
     </row>
@@ -7380,7 +7315,6 @@
       <c r="E66" t="s">
         <v>248</v>
       </c>
-      <c r="G66" s="103"/>
       <c r="J66" s="101"/>
       <c r="Q66" s="57"/>
     </row>
@@ -7400,7 +7334,6 @@
       <c r="E67" t="s">
         <v>248</v>
       </c>
-      <c r="G67" s="103"/>
       <c r="J67" s="101"/>
       <c r="Q67" s="57"/>
     </row>
@@ -7420,7 +7353,6 @@
       <c r="E68" t="s">
         <v>248</v>
       </c>
-      <c r="G68" s="103"/>
       <c r="J68" s="101"/>
       <c r="Q68" s="57"/>
     </row>
@@ -7440,7 +7372,6 @@
       <c r="E69" t="s">
         <v>248</v>
       </c>
-      <c r="G69" s="103"/>
       <c r="J69" s="101"/>
       <c r="Q69" s="57"/>
     </row>
@@ -7460,7 +7391,6 @@
       <c r="E70" t="s">
         <v>248</v>
       </c>
-      <c r="G70" s="103"/>
       <c r="J70" s="101"/>
       <c r="Q70" s="57"/>
     </row>
@@ -7480,7 +7410,6 @@
       <c r="E71" t="s">
         <v>248</v>
       </c>
-      <c r="G71" s="103"/>
       <c r="J71" s="101"/>
       <c r="Q71" s="57"/>
     </row>
@@ -7500,7 +7429,6 @@
       <c r="E72" t="s">
         <v>248</v>
       </c>
-      <c r="G72" s="103"/>
       <c r="J72" s="101"/>
       <c r="Q72" s="57"/>
     </row>
@@ -7520,7 +7448,6 @@
       <c r="E73" t="s">
         <v>248</v>
       </c>
-      <c r="G73" s="103"/>
       <c r="J73" s="101"/>
       <c r="Q73" s="57"/>
     </row>
@@ -7540,7 +7467,6 @@
       <c r="E74" t="s">
         <v>248</v>
       </c>
-      <c r="G74" s="103"/>
       <c r="J74" s="101"/>
       <c r="Q74" s="57"/>
     </row>
@@ -7560,7 +7486,6 @@
       <c r="E75" t="s">
         <v>248</v>
       </c>
-      <c r="G75" s="103"/>
       <c r="J75" s="101"/>
     </row>
     <row r="76" spans="1:17">
@@ -7579,7 +7504,6 @@
       <c r="E76" t="s">
         <v>247</v>
       </c>
-      <c r="G76" s="103"/>
       <c r="J76" s="101"/>
     </row>
     <row r="77" spans="1:17">
@@ -7598,7 +7522,6 @@
       <c r="E77" t="s">
         <v>248</v>
       </c>
-      <c r="G77" s="103"/>
       <c r="J77" s="101"/>
     </row>
     <row r="78" spans="1:17">
@@ -7617,7 +7540,6 @@
       <c r="E78" t="s">
         <v>248</v>
       </c>
-      <c r="G78" s="103"/>
       <c r="J78" s="101"/>
     </row>
     <row r="79" spans="1:17">
@@ -7636,7 +7558,6 @@
       <c r="E79" t="s">
         <v>248</v>
       </c>
-      <c r="G79" s="103"/>
       <c r="J79" s="101"/>
     </row>
     <row r="80" spans="1:17">
@@ -7655,7 +7576,6 @@
       <c r="E80" t="s">
         <v>248</v>
       </c>
-      <c r="G80" s="103"/>
       <c r="J80" s="101"/>
     </row>
     <row r="81" spans="1:15">
@@ -7674,7 +7594,6 @@
       <c r="E81" t="s">
         <v>248</v>
       </c>
-      <c r="G81" s="103"/>
       <c r="J81" s="101"/>
       <c r="K81" s="57"/>
     </row>
@@ -7694,7 +7613,6 @@
       <c r="E82" t="s">
         <v>248</v>
       </c>
-      <c r="G82" s="103"/>
       <c r="J82" s="101"/>
       <c r="K82" s="57"/>
     </row>
@@ -7714,7 +7632,6 @@
       <c r="E83" t="s">
         <v>248</v>
       </c>
-      <c r="G83" s="103"/>
       <c r="J83" s="101"/>
       <c r="K83" s="57"/>
     </row>
@@ -7734,7 +7651,6 @@
       <c r="E84" t="s">
         <v>248</v>
       </c>
-      <c r="G84" s="103"/>
       <c r="J84" s="101"/>
       <c r="K84" s="57"/>
     </row>
@@ -7754,7 +7670,6 @@
       <c r="E85" t="s">
         <v>248</v>
       </c>
-      <c r="G85" s="103"/>
       <c r="J85" s="101"/>
       <c r="K85" s="57"/>
     </row>
@@ -7774,7 +7689,6 @@
       <c r="E86" t="s">
         <v>248</v>
       </c>
-      <c r="G86" s="103"/>
       <c r="J86" s="101"/>
       <c r="K86" s="57"/>
     </row>
@@ -7794,7 +7708,6 @@
       <c r="E87" t="s">
         <v>248</v>
       </c>
-      <c r="G87" s="103"/>
       <c r="J87" s="101"/>
       <c r="K87" s="57"/>
     </row>
@@ -7814,7 +7727,6 @@
       <c r="E88" t="s">
         <v>247</v>
       </c>
-      <c r="G88" s="103"/>
       <c r="J88" s="101"/>
       <c r="K88" s="57"/>
     </row>
@@ -7834,7 +7746,6 @@
       <c r="E89" t="s">
         <v>248</v>
       </c>
-      <c r="G89" s="103"/>
       <c r="J89" s="101"/>
       <c r="K89" s="57"/>
     </row>
@@ -7854,7 +7765,6 @@
       <c r="E90" t="s">
         <v>248</v>
       </c>
-      <c r="G90" s="103"/>
       <c r="J90" s="101"/>
       <c r="K90" s="57"/>
     </row>
@@ -7874,7 +7784,6 @@
       <c r="E91" t="s">
         <v>248</v>
       </c>
-      <c r="G91" s="103"/>
       <c r="J91" s="101"/>
       <c r="K91" s="57"/>
       <c r="N91" s="57"/>
@@ -7896,7 +7805,6 @@
       <c r="E92" t="s">
         <v>248</v>
       </c>
-      <c r="G92" s="103"/>
       <c r="J92" s="101"/>
       <c r="K92" s="57"/>
       <c r="N92" s="57"/>
@@ -7918,7 +7826,6 @@
       <c r="E93" t="s">
         <v>248</v>
       </c>
-      <c r="G93" s="103"/>
       <c r="J93" s="101"/>
       <c r="N93" s="57"/>
       <c r="O93" s="1"/>
@@ -7939,7 +7846,6 @@
       <c r="E94" t="s">
         <v>248</v>
       </c>
-      <c r="G94" s="103"/>
       <c r="J94" s="101"/>
       <c r="N94" s="57"/>
       <c r="O94" s="1"/>
@@ -7960,7 +7866,6 @@
       <c r="E95" t="s">
         <v>248</v>
       </c>
-      <c r="G95" s="103"/>
       <c r="J95" s="101"/>
       <c r="N95" s="57"/>
       <c r="O95" s="1"/>
@@ -7981,7 +7886,6 @@
       <c r="E96" t="s">
         <v>248</v>
       </c>
-      <c r="G96" s="103"/>
       <c r="J96" s="101"/>
       <c r="N96" s="57"/>
       <c r="O96" s="1"/>
@@ -8002,7 +7906,6 @@
       <c r="E97" t="s">
         <v>248</v>
       </c>
-      <c r="G97" s="103"/>
       <c r="J97" s="101"/>
       <c r="N97" s="57"/>
       <c r="O97" s="1"/>
@@ -8023,7 +7926,6 @@
       <c r="E98" t="s">
         <v>248</v>
       </c>
-      <c r="G98" s="103"/>
       <c r="J98" s="101"/>
       <c r="N98" s="57"/>
       <c r="O98" s="1"/>
@@ -8044,7 +7946,6 @@
       <c r="E99" t="s">
         <v>248</v>
       </c>
-      <c r="G99" s="103"/>
       <c r="J99" s="101"/>
       <c r="N99" s="57"/>
     </row>
@@ -8064,7 +7965,6 @@
       <c r="E100" t="s">
         <v>247</v>
       </c>
-      <c r="G100" s="103"/>
       <c r="J100" s="101"/>
       <c r="N100" s="57"/>
     </row>
@@ -8084,7 +7984,6 @@
       <c r="E101" t="s">
         <v>248</v>
       </c>
-      <c r="G101" s="103"/>
       <c r="J101" s="101"/>
       <c r="N101" s="57"/>
     </row>
@@ -8104,7 +8003,6 @@
       <c r="E102" t="s">
         <v>248</v>
       </c>
-      <c r="G102" s="103"/>
       <c r="J102" s="101"/>
       <c r="N102" s="57"/>
     </row>
@@ -8124,7 +8022,6 @@
       <c r="E103" t="s">
         <v>248</v>
       </c>
-      <c r="G103" s="103"/>
       <c r="J103" s="101"/>
     </row>
     <row r="104" spans="1:15">
@@ -8143,7 +8040,6 @@
       <c r="E104" t="s">
         <v>248</v>
       </c>
-      <c r="G104" s="103"/>
       <c r="J104" s="101"/>
     </row>
     <row r="105" spans="1:15">
@@ -8157,12 +8053,11 @@
         <v>46113</v>
       </c>
       <c r="D105">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E105" t="s">
         <v>248</v>
       </c>
-      <c r="G105" s="103"/>
       <c r="J105" s="101"/>
     </row>
     <row r="106" spans="1:15">
@@ -8181,7 +8076,6 @@
       <c r="E106" t="s">
         <v>248</v>
       </c>
-      <c r="G106" s="103"/>
       <c r="J106" s="101"/>
     </row>
     <row r="107" spans="1:15">
@@ -8200,7 +8094,6 @@
       <c r="E107" t="s">
         <v>248</v>
       </c>
-      <c r="G107" s="103"/>
       <c r="J107" s="101"/>
     </row>
     <row r="108" spans="1:15">
@@ -8219,7 +8112,6 @@
       <c r="E108" t="s">
         <v>248</v>
       </c>
-      <c r="G108" s="103"/>
       <c r="J108" s="101"/>
     </row>
     <row r="109" spans="1:15">
@@ -8238,7 +8130,6 @@
       <c r="E109" t="s">
         <v>248</v>
       </c>
-      <c r="G109" s="103"/>
       <c r="J109" s="101"/>
     </row>
     <row r="110" spans="1:15">
@@ -8257,7 +8148,6 @@
       <c r="E110" t="s">
         <v>248</v>
       </c>
-      <c r="G110" s="103"/>
       <c r="J110" s="101"/>
     </row>
     <row r="111" spans="1:15">
@@ -8276,7 +8166,6 @@
       <c r="E111" t="s">
         <v>248</v>
       </c>
-      <c r="G111" s="103"/>
       <c r="J111" s="101"/>
     </row>
     <row r="112" spans="1:15">
@@ -8295,7 +8184,6 @@
       <c r="E112" t="s">
         <v>247</v>
       </c>
-      <c r="G112" s="103"/>
       <c r="J112" s="101"/>
     </row>
     <row r="113" spans="1:11">
@@ -8314,7 +8202,6 @@
       <c r="E113" t="s">
         <v>248</v>
       </c>
-      <c r="G113" s="103"/>
       <c r="J113" s="101"/>
       <c r="K113" s="57"/>
     </row>
@@ -8334,7 +8221,6 @@
       <c r="E114" t="s">
         <v>248</v>
       </c>
-      <c r="G114" s="103"/>
       <c r="J114" s="101"/>
       <c r="K114" s="57"/>
     </row>
@@ -8354,7 +8240,6 @@
       <c r="E115" t="s">
         <v>248</v>
       </c>
-      <c r="G115" s="103"/>
       <c r="J115" s="101"/>
       <c r="K115" s="57"/>
     </row>
@@ -8374,7 +8259,6 @@
       <c r="E116" t="s">
         <v>248</v>
       </c>
-      <c r="G116" s="103"/>
       <c r="J116" s="101"/>
       <c r="K116" s="57"/>
     </row>
@@ -8394,7 +8278,6 @@
       <c r="E117" t="s">
         <v>248</v>
       </c>
-      <c r="G117" s="103"/>
       <c r="J117" s="101"/>
       <c r="K117" s="57"/>
     </row>
@@ -8414,7 +8297,6 @@
       <c r="E118" t="s">
         <v>248</v>
       </c>
-      <c r="G118" s="103"/>
       <c r="J118" s="101"/>
       <c r="K118" s="57"/>
     </row>
@@ -8434,7 +8316,6 @@
       <c r="E119" t="s">
         <v>248</v>
       </c>
-      <c r="G119" s="103"/>
       <c r="J119" s="101"/>
       <c r="K119" s="57"/>
     </row>
@@ -8454,7 +8335,6 @@
       <c r="E120" t="s">
         <v>248</v>
       </c>
-      <c r="G120" s="103"/>
       <c r="J120" s="101"/>
       <c r="K120" s="57"/>
     </row>
@@ -8474,7 +8354,6 @@
       <c r="E121" t="s">
         <v>248</v>
       </c>
-      <c r="G121" s="103"/>
       <c r="J121" s="101"/>
       <c r="K121" s="57"/>
     </row>
@@ -8498,22 +8377,22 @@
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2C43C22-3382-D94C-AF1F-BAB48F8FB89E}">
   <dimension ref="A1:X33"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
+  <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
   <cols>
     <col min="1" max="1" width="3.75" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="46.375" customWidth="1"/>
-    <col min="3" max="3" width="60.375" customWidth="1"/>
+    <col min="2" max="2" width="46.33203125" customWidth="1"/>
+    <col min="3" max="3" width="60.33203125" customWidth="1"/>
     <col min="4" max="4" width="61" customWidth="1"/>
-    <col min="5" max="5" width="33.875" customWidth="1"/>
-    <col min="6" max="6" width="20.875" customWidth="1"/>
-    <col min="7" max="18" width="13.875" customWidth="1"/>
-    <col min="19" max="19" width="31.625" customWidth="1"/>
+    <col min="5" max="5" width="33.83203125" customWidth="1"/>
+    <col min="6" max="6" width="20.83203125" customWidth="1"/>
+    <col min="7" max="18" width="13.83203125" customWidth="1"/>
+    <col min="19" max="19" width="31.58203125" customWidth="1"/>
     <col min="20" max="20" width="18" customWidth="1"/>
-    <col min="21" max="21" width="15.125" customWidth="1"/>
-    <col min="22" max="22" width="63.125" customWidth="1"/>
+    <col min="21" max="21" width="15.08203125" customWidth="1"/>
+    <col min="22" max="22" width="63.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:24" s="49" customFormat="1" ht="54">
+    <row r="1" spans="1:24" s="49" customFormat="1" ht="52.5">
       <c r="A1" s="45" t="s">
         <v>0</v>
       </c>
@@ -8585,7 +8464,7 @@
         <v>0.66666666666666663</v>
       </c>
     </row>
-    <row r="2" spans="1:24" ht="30.75">
+    <row r="2" spans="1:24" ht="31">
       <c r="A2" s="33">
         <v>1</v>
       </c>
@@ -8639,7 +8518,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:24">
+    <row r="3" spans="1:24" ht="16">
       <c r="A3" s="34">
         <v>2</v>
       </c>
@@ -8685,7 +8564,7 @@
       </c>
       <c r="V3" s="17"/>
     </row>
-    <row r="4" spans="1:24" ht="60">
+    <row r="4" spans="1:24" ht="75">
       <c r="A4" s="33">
         <v>3</v>
       </c>
@@ -8812,7 +8691,7 @@
       </c>
       <c r="V5" s="18"/>
     </row>
-    <row r="6" spans="1:24" ht="75">
+    <row r="6" spans="1:24" ht="90">
       <c r="A6" s="36">
         <v>5</v>
       </c>
@@ -8890,7 +8769,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="7" spans="1:24" ht="56.1" customHeight="1">
+    <row r="7" spans="1:24" ht="56.15" customHeight="1">
       <c r="A7" s="35">
         <v>6</v>
       </c>
@@ -8962,7 +8841,7 @@
         <v>23</v>
       </c>
     </row>
-    <row r="8" spans="1:24" ht="56.1" customHeight="1">
+    <row r="8" spans="1:24" ht="56.15" customHeight="1">
       <c r="A8" s="36">
         <v>7</v>
       </c>
@@ -9034,7 +8913,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="9" spans="1:24" ht="30">
+    <row r="9" spans="1:24" ht="45">
       <c r="A9" s="35">
         <v>8</v>
       </c>
@@ -9103,7 +8982,7 @@
       </c>
       <c r="V9" s="18"/>
     </row>
-    <row r="10" spans="1:24" ht="30">
+    <row r="10" spans="1:24" ht="45">
       <c r="A10" s="36">
         <v>9</v>
       </c>
@@ -9239,59 +9118,59 @@
       </c>
       <c r="V11" s="18"/>
     </row>
-    <row r="13" spans="1:24">
+    <row r="13" spans="1:24" ht="16">
       <c r="T13" s="4"/>
     </row>
-    <row r="14" spans="1:24">
+    <row r="14" spans="1:24" ht="16">
       <c r="T14" s="4"/>
     </row>
-    <row r="15" spans="1:24">
+    <row r="15" spans="1:24" ht="16">
       <c r="C15" t="s">
         <v>32</v>
       </c>
       <c r="T15" s="5"/>
     </row>
-    <row r="16" spans="1:24">
+    <row r="16" spans="1:24" ht="16">
       <c r="C16" t="s">
         <v>33</v>
       </c>
       <c r="T16" s="6"/>
     </row>
-    <row r="17" spans="6:20">
+    <row r="17" spans="6:20" ht="16">
       <c r="F17" s="3"/>
       <c r="T17" s="5"/>
     </row>
-    <row r="18" spans="6:20">
+    <row r="18" spans="6:20" ht="16">
       <c r="T18" s="6"/>
     </row>
-    <row r="19" spans="6:20">
+    <row r="19" spans="6:20" ht="16">
       <c r="T19" s="5"/>
     </row>
-    <row r="20" spans="6:20">
+    <row r="20" spans="6:20" ht="16">
       <c r="T20" s="6"/>
     </row>
-    <row r="21" spans="6:20">
+    <row r="21" spans="6:20" ht="16">
       <c r="T21" s="5"/>
     </row>
-    <row r="22" spans="6:20">
+    <row r="22" spans="6:20" ht="16">
       <c r="T22" s="6"/>
     </row>
-    <row r="23" spans="6:20">
+    <row r="23" spans="6:20" ht="16">
       <c r="T23" s="2"/>
     </row>
-    <row r="24" spans="6:20">
+    <row r="24" spans="6:20" ht="16">
       <c r="T24" s="4"/>
     </row>
-    <row r="25" spans="6:20">
+    <row r="25" spans="6:20" ht="16">
       <c r="T25" s="4"/>
     </row>
-    <row r="26" spans="6:20">
+    <row r="26" spans="6:20" ht="16">
       <c r="T26" s="4"/>
     </row>
-    <row r="27" spans="6:20">
+    <row r="27" spans="6:20" ht="16">
       <c r="T27" s="4"/>
     </row>
-    <row r="28" spans="6:20">
+    <row r="28" spans="6:20" ht="16">
       <c r="T28" s="4"/>
     </row>
     <row r="33" spans="10:10" ht="15.75" customHeight="1">
@@ -9503,6 +9382,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010067C3E934A0AA0B40A01BB34EE44DBE4E" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="99f90e1838b691a269ec0be7c9d3b1c4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7bc4fa38-d888-4f67-9acc-d35155363a39" xmlns:ns3="fff59cbe-7145-45c6-b0b8-a33a9ec94a75" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="55b527a863acd720578db25cd4da17b2" ns2:_="" ns3:_="">
     <xsd:import namespace="7bc4fa38-d888-4f67-9acc-d35155363a39"/>
@@ -9697,15 +9585,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9F09B98-3A3F-4A19-9439-839483AD047D}">
   <ds:schemaRefs>
@@ -9724,6 +9603,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57AD8670-20BC-4534-A7A5-87984349E00F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{339BB920-340D-4757-A55F-4B7C981C835F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9740,12 +9627,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57AD8670-20BC-4534-A7A5-87984349E00F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
refactor(model, dax): flatten kpis dimension and streamline Adjusted_Target_Value
Removed the snowflake 'units' table and integrated Target_Unit and Actual_Unit directly into the 'kpis' dimension to optimize the Star Schema. Refactored the DAX measure to read units directly from the KPI context, maintaining the dynamic Relative Growth vs Absolute Target logic with improved query performance.
</commit_message>
<xml_diff>
--- a/Datasets/okrs.xlsx
+++ b/Datasets/okrs.xlsx
@@ -8,26 +8,25 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauro.turner\Proyectos\Dashboards\Global-IT---OKR-KPI-Dashboard\Datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C0D0F15-C948-4C6A-8A14-6A59F7FA4593}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8331B162-FE24-49B7-8074-6047397F3554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="810" activeTab="7" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="810" firstSheet="1" activeTab="3" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
   </bookViews>
   <sheets>
     <sheet name="objetives" sheetId="11" r:id="rId1"/>
     <sheet name="owners" sheetId="14" r:id="rId2"/>
     <sheet name="sources" sheetId="15" r:id="rId3"/>
-    <sheet name="units" sheetId="16" r:id="rId4"/>
-    <sheet name="kpis" sheetId="13" r:id="rId5"/>
-    <sheet name="kpi_owners" sheetId="17" r:id="rId6"/>
-    <sheet name="kpi_sources" sheetId="18" r:id="rId7"/>
-    <sheet name="Results" sheetId="19" r:id="rId8"/>
-    <sheet name="GLOBAL IT OKRs " sheetId="1" r:id="rId9"/>
-    <sheet name="1- AI Skills Workday" sheetId="5" r:id="rId10"/>
-    <sheet name="2- AI TQ Courses" sheetId="6" r:id="rId11"/>
-    <sheet name="3- AI-related Learning Events" sheetId="7" r:id="rId12"/>
-    <sheet name="5-Engagement events" sheetId="8" r:id="rId13"/>
-    <sheet name="6-Monthly Campaings (VE)" sheetId="9" r:id="rId14"/>
-    <sheet name="7-Career Worth" sheetId="10" r:id="rId15"/>
+    <sheet name="kpis" sheetId="13" r:id="rId4"/>
+    <sheet name="kpi_owners" sheetId="17" r:id="rId5"/>
+    <sheet name="kpi_sources" sheetId="18" r:id="rId6"/>
+    <sheet name="Results" sheetId="19" r:id="rId7"/>
+    <sheet name="GLOBAL IT OKRs " sheetId="1" r:id="rId8"/>
+    <sheet name="1- AI Skills Workday" sheetId="5" r:id="rId9"/>
+    <sheet name="2- AI TQ Courses" sheetId="6" r:id="rId10"/>
+    <sheet name="3- AI-related Learning Events" sheetId="7" r:id="rId11"/>
+    <sheet name="5-Engagement events" sheetId="8" r:id="rId12"/>
+    <sheet name="6-Monthly Campaings (VE)" sheetId="9" r:id="rId13"/>
+    <sheet name="7-Career Worth" sheetId="10" r:id="rId14"/>
   </sheets>
   <calcPr calcId="191028"/>
   <extLst>
@@ -78,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="528" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="250">
   <si>
     <t>ID</t>
   </si>
@@ -1259,12 +1258,6 @@
     <t>Engagement Team</t>
   </si>
   <si>
-    <t>Unit_ID</t>
-  </si>
-  <si>
-    <t>Unit_Name</t>
-  </si>
-  <si>
     <t>Percentage</t>
   </si>
   <si>
@@ -1290,6 +1283,12 @@
   </si>
   <si>
     <t>sep-25</t>
+  </si>
+  <si>
+    <t>Actual_Unit</t>
+  </si>
+  <si>
+    <t>Target_Unit</t>
   </si>
 </sst>
 </file>
@@ -1300,7 +1299,7 @@
     <numFmt numFmtId="164" formatCode="m/d/yy;@"/>
     <numFmt numFmtId="165" formatCode="[$-1540A]m/d/yyyy;@"/>
   </numFmts>
-  <fonts count="32">
+  <fonts count="31">
     <font>
       <sz val="12"/>
       <color theme="1"/>
@@ -1493,14 +1492,6 @@
       <color rgb="FF464FEB"/>
       <name val="Segoe UI"/>
       <family val="2"/>
-    </font>
-    <font>
-      <b/>
-      <sz val="12"/>
-      <color theme="0"/>
-      <name val="Aptos Narrow"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="11">
@@ -1718,7 +1709,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="103">
+  <cellXfs count="100">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="9" fontId="2" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
@@ -1983,9 +1974,6 @@
     <xf numFmtId="9" fontId="3" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="31" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
@@ -1993,7 +1981,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="26">
+  <dxfs count="24">
     <dxf>
       <font>
         <strike val="0"/>
@@ -2376,46 +2364,6 @@
     </dxf>
     <dxf>
       <numFmt numFmtId="165" formatCode="[$-1540A]m/d/yyyy;@"/>
-    </dxf>
-    <dxf>
-      <border outline="0">
-        <left style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </left>
-        <right style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </right>
-        <top style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </top>
-        <bottom style="thin">
-          <color theme="4" tint="0.39997558519241921"/>
-        </bottom>
-      </border>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-        <strike val="0"/>
-        <condense val="0"/>
-        <extend val="0"/>
-        <outline val="0"/>
-        <shadow val="0"/>
-        <u val="none"/>
-        <vertAlign val="baseline"/>
-        <sz val="12"/>
-        <color theme="0"/>
-        <name val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </font>
-      <fill>
-        <patternFill patternType="solid">
-          <fgColor theme="4"/>
-          <bgColor theme="4"/>
-        </patternFill>
-      </fill>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -3062,23 +3010,13 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{6AAE90B7-0747-44B6-892C-5C0FB09C6261}" name="units" displayName="units" ref="A1:B3" totalsRowShown="0" headerRowDxfId="25" tableBorderDxfId="24">
-  <autoFilter ref="A1:B3" xr:uid="{6AAE90B7-0747-44B6-892C-5C0FB09C6261}"/>
-  <tableColumns count="2">
-    <tableColumn id="1" xr3:uid="{78A9EFFF-8B69-456A-BE78-36EE4A6917F7}" name="Unit_ID"/>
-    <tableColumn id="2" xr3:uid="{AC9CF5AF-7CCA-440B-9A30-C4372D1D43D7}" name="Unit_Name"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
-</file>
-
-<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{05CF7CEB-E38D-4385-9D0A-7780DBE1F2C6}" name="kpis" displayName="kpis" ref="A1:E11" totalsRowShown="0">
-  <autoFilter ref="A1:E11" xr:uid="{05CF7CEB-E38D-4385-9D0A-7780DBE1F2C6}"/>
-  <tableColumns count="5">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{05CF7CEB-E38D-4385-9D0A-7780DBE1F2C6}" name="kpis" displayName="kpis" ref="A1:F11" totalsRowShown="0">
+  <autoFilter ref="A1:F11" xr:uid="{05CF7CEB-E38D-4385-9D0A-7780DBE1F2C6}"/>
+  <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{68ECD000-5CB1-4C4B-BB03-A6A5B1FE144C}" name="KPI_ID"/>
     <tableColumn id="2" xr3:uid="{EE4E4C8E-E234-462A-B525-6959D9606CDE}" name="Objetive_ID"/>
-    <tableColumn id="3" xr3:uid="{46D9FC96-8D58-4277-8E94-058CE19E84BF}" name="Unit_ID"/>
+    <tableColumn id="6" xr3:uid="{AC2714AF-A87A-4389-91F0-B64D137D4FCB}" name="Target_Unit"/>
+    <tableColumn id="3" xr3:uid="{46D9FC96-8D58-4277-8E94-058CE19E84BF}" name="Actual_Unit"/>
     <tableColumn id="4" xr3:uid="{F5A9C9F6-F438-47DA-A6B5-34F34C02DBAD}" name="KPI_Goal"/>
     <tableColumn id="5" xr3:uid="{E5AD5A19-0EBD-4165-9D29-1E69182B7E49}" name="Target_Value"/>
   </tableColumns>
@@ -3086,7 +3024,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table5.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="6" xr:uid="{0665482D-6BB4-4BFD-8C37-E470C73D1B9E}" name="kpi_owners" displayName="kpi_owners" ref="A1:B15" totalsRowShown="0">
   <autoFilter ref="A1:B15" xr:uid="{0665482D-6BB4-4BFD-8C37-E470C73D1B9E}"/>
   <tableColumns count="2">
@@ -3097,7 +3035,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table6.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="7" xr:uid="{CFAAFB16-B748-431B-BE7F-496A57C5D8BD}" name="kpi_sources" displayName="kpi_sources" ref="A1:B15" totalsRowShown="0">
   <autoFilter ref="A1:B15" xr:uid="{CFAAFB16-B748-431B-BE7F-496A57C5D8BD}"/>
   <tableColumns count="2">
@@ -3108,7 +3046,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table7.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="8" xr:uid="{F5D35D80-1415-4E63-ABD5-5C8B2EFFCF70}" name="results" displayName="results" ref="A1:E121" totalsRowShown="0">
   <autoFilter ref="A1:E121" xr:uid="{F5D35D80-1415-4E63-ABD5-5C8B2EFFCF70}"/>
   <tableColumns count="5">
@@ -3122,7 +3060,7 @@
 </table>
 </file>
 
-<file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/tables/table8.xml><?xml version="1.0" encoding="utf-8"?>
 <table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{ADB8C96C-1591-5F48-A392-4D1EC7052CD5}" name="Table1" displayName="Table1" ref="B1:V11" totalsRowShown="0" headerRowDxfId="22" dataDxfId="21">
   <autoFilter ref="B1:V11" xr:uid="{ADB8C96C-1591-5F48-A392-4D1EC7052CD5}"/>
   <tableColumns count="21">
@@ -3532,88 +3470,6 @@
 </file>
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A1C2DE-958E-4EF5-BD32-D7572A596892}">
-  <dimension ref="A1:C81"/>
-  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
-  <sheetData>
-    <row r="1" spans="1:1">
-      <c r="A1" s="57">
-        <v>46062</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3">
-      <c r="A17">
-        <v>5911</v>
-      </c>
-      <c r="B17">
-        <v>3758</v>
-      </c>
-      <c r="C17" s="58">
-        <f>+B17/A17</f>
-        <v>0.63576383014718318</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3">
-      <c r="B18">
-        <v>986</v>
-      </c>
-      <c r="C18" s="58">
-        <f>+B18/A17</f>
-        <v>0.16680764676027746</v>
-      </c>
-    </row>
-    <row r="42" spans="1:1">
-      <c r="A42" s="57">
-        <v>46085</v>
-      </c>
-    </row>
-    <row r="69" spans="1:1">
-      <c r="A69" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="70" spans="1:1">
-      <c r="A70">
-        <v>5943</v>
-      </c>
-    </row>
-    <row r="72" spans="1:1">
-      <c r="A72" t="s">
-        <v>209</v>
-      </c>
-    </row>
-    <row r="73" spans="1:1">
-      <c r="A73">
-        <v>5258</v>
-      </c>
-    </row>
-    <row r="75" spans="1:1">
-      <c r="A75" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="76" spans="1:1">
-      <c r="A76">
-        <v>5101</v>
-      </c>
-    </row>
-    <row r="80" spans="1:1">
-      <c r="A80" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="81" spans="1:1">
-      <c r="A81">
-        <v>4884</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <drawing r:id="rId1"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6A5511CF-ECA4-4801-B421-12A212CAD755}">
   <dimension ref="A1:R81"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
@@ -4146,7 +4002,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4BAD0912-E0CB-460C-ABF0-F667933348DC}">
   <dimension ref="A1:B7"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
@@ -4208,7 +4064,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FECA49D2-6EDF-4BD1-9DAB-FC593DCBD3BD}">
   <dimension ref="A2:H78"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
@@ -5284,7 +5140,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{92D61564-BD00-449F-B779-9A392A403D13}">
   <dimension ref="A2:A14"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
@@ -5349,7 +5205,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B73C4F58-E1C8-4D89-93FA-19463BA41BD4}">
   <dimension ref="A1:A3"/>
   <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
@@ -5567,35 +5423,225 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78397758-3182-4D2B-AEC2-12D8A685B44A}">
-  <dimension ref="A1:B3"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5716ADCC-E36E-44A5-AF6D-43063C282787}">
+  <dimension ref="A1:F11"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
-    <col min="2" max="2" width="11.75" customWidth="1"/>
+    <col min="2" max="3" width="12.08203125" customWidth="1"/>
+    <col min="4" max="4" width="12.6640625" customWidth="1"/>
+    <col min="5" max="5" width="29.5" customWidth="1"/>
+    <col min="6" max="6" width="13.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" s="99" t="s">
+    <row r="1" spans="1:6">
+      <c r="A1" t="s">
+        <v>214</v>
+      </c>
+      <c r="B1" t="s">
+        <v>212</v>
+      </c>
+      <c r="C1" t="s">
+        <v>249</v>
+      </c>
+      <c r="D1" t="s">
+        <v>248</v>
+      </c>
+      <c r="E1" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6">
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2">
+        <v>1</v>
+      </c>
+      <c r="C2" t="s">
         <v>239</v>
       </c>
-      <c r="B1" s="99" t="s">
+      <c r="D2" t="s">
         <v>240</v>
       </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2" s="98">
+      <c r="E2" t="s">
+        <v>34</v>
+      </c>
+      <c r="F2">
+        <v>0.2</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6">
+      <c r="A3">
+        <v>2</v>
+      </c>
+      <c r="B3">
         <v>1</v>
       </c>
-      <c r="B2" s="98" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3" s="100">
+      <c r="C3" t="s">
+        <v>239</v>
+      </c>
+      <c r="D3" t="s">
+        <v>239</v>
+      </c>
+      <c r="E3" t="s">
+        <v>36</v>
+      </c>
+      <c r="F3">
+        <v>0.7</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6">
+      <c r="A4">
+        <v>3</v>
+      </c>
+      <c r="B4">
+        <v>1</v>
+      </c>
+      <c r="C4" t="s">
+        <v>240</v>
+      </c>
+      <c r="D4" t="s">
+        <v>240</v>
+      </c>
+      <c r="E4" t="s">
+        <v>16</v>
+      </c>
+      <c r="F4">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6">
+      <c r="A5">
+        <v>4</v>
+      </c>
+      <c r="B5">
         <v>2</v>
       </c>
-      <c r="B3" s="100" t="s">
-        <v>242</v>
+      <c r="C5" t="s">
+        <v>240</v>
+      </c>
+      <c r="D5" t="s">
+        <v>240</v>
+      </c>
+      <c r="E5" t="s">
+        <v>18</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6">
+      <c r="A6">
+        <v>5</v>
+      </c>
+      <c r="B6">
+        <v>2</v>
+      </c>
+      <c r="C6" t="s">
+        <v>240</v>
+      </c>
+      <c r="D6" t="s">
+        <v>240</v>
+      </c>
+      <c r="E6" t="s">
+        <v>19</v>
+      </c>
+      <c r="F6">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6">
+      <c r="A7">
+        <v>6</v>
+      </c>
+      <c r="B7">
+        <v>2</v>
+      </c>
+      <c r="C7" t="s">
+        <v>240</v>
+      </c>
+      <c r="D7" t="s">
+        <v>240</v>
+      </c>
+      <c r="E7" t="s">
+        <v>21</v>
+      </c>
+      <c r="F7">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6">
+      <c r="A8">
+        <v>7</v>
+      </c>
+      <c r="B8">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
+        <v>240</v>
+      </c>
+      <c r="D8" t="s">
+        <v>240</v>
+      </c>
+      <c r="E8" t="s">
+        <v>25</v>
+      </c>
+      <c r="F8">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6">
+      <c r="A9">
+        <v>8</v>
+      </c>
+      <c r="B9">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
+        <v>239</v>
+      </c>
+      <c r="D9" t="s">
+        <v>239</v>
+      </c>
+      <c r="E9" t="s">
+        <v>27</v>
+      </c>
+      <c r="F9">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6">
+      <c r="A10">
+        <v>9</v>
+      </c>
+      <c r="B10">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
+        <v>240</v>
+      </c>
+      <c r="D10" t="s">
+        <v>240</v>
+      </c>
+      <c r="E10" t="s">
+        <v>29</v>
+      </c>
+      <c r="F10">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6">
+      <c r="A11">
+        <v>10</v>
+      </c>
+      <c r="B11">
+        <v>3</v>
+      </c>
+      <c r="E11" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -5607,194 +5653,128 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5716ADCC-E36E-44A5-AF6D-43063C282787}">
-  <dimension ref="A1:E11"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3992BCCC-153D-40F1-88B0-57A653F9FE93}">
+  <dimension ref="A1:B15"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
-  <cols>
-    <col min="2" max="2" width="12.08203125" customWidth="1"/>
-    <col min="4" max="4" width="29.5" customWidth="1"/>
-    <col min="5" max="5" width="13.08203125" customWidth="1"/>
-  </cols>
   <sheetData>
-    <row r="1" spans="1:5">
+    <row r="1" spans="1:2">
       <c r="A1" t="s">
         <v>214</v>
       </c>
       <c r="B1" t="s">
-        <v>212</v>
-      </c>
-      <c r="C1" t="s">
-        <v>239</v>
-      </c>
-      <c r="D1" t="s">
-        <v>215</v>
-      </c>
-      <c r="E1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="2" spans="1:5">
+        <v>228</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2">
       <c r="A2">
         <v>1</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2">
-        <v>1</v>
-      </c>
-      <c r="D2" t="s">
-        <v>34</v>
-      </c>
-      <c r="E2">
-        <v>0.2</v>
-      </c>
-    </row>
-    <row r="3" spans="1:5">
+    </row>
+    <row r="3" spans="1:2">
       <c r="A3">
         <v>2</v>
       </c>
       <c r="B3">
-        <v>1</v>
-      </c>
-      <c r="C3">
-        <v>1</v>
-      </c>
-      <c r="D3" t="s">
-        <v>36</v>
-      </c>
-      <c r="E3">
-        <v>0.7</v>
-      </c>
-    </row>
-    <row r="4" spans="1:5">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="4" spans="1:2">
       <c r="A4">
         <v>3</v>
       </c>
       <c r="B4">
-        <v>1</v>
-      </c>
-      <c r="C4">
-        <v>2</v>
-      </c>
-      <c r="D4" t="s">
-        <v>16</v>
-      </c>
-      <c r="E4">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="5" spans="1:5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" spans="1:2">
       <c r="A5">
+        <v>3</v>
+      </c>
+      <c r="B5">
         <v>4</v>
       </c>
-      <c r="B5">
-        <v>2</v>
-      </c>
-      <c r="C5">
-        <v>2</v>
-      </c>
-      <c r="D5" t="s">
-        <v>18</v>
-      </c>
-      <c r="E5">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="6" spans="1:5">
+    </row>
+    <row r="6" spans="1:2">
       <c r="A6">
+        <v>4</v>
+      </c>
+      <c r="B6">
         <v>5</v>
       </c>
-      <c r="B6">
-        <v>2</v>
-      </c>
-      <c r="C6">
-        <v>2</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="7" spans="1:5">
+    </row>
+    <row r="7" spans="1:2">
       <c r="A7">
+        <v>4</v>
+      </c>
+      <c r="B7">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:2">
+      <c r="A8">
+        <v>5</v>
+      </c>
+      <c r="B8">
         <v>6</v>
       </c>
-      <c r="B7">
-        <v>2</v>
-      </c>
-      <c r="C7">
-        <v>2</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="8" spans="1:5">
-      <c r="A8">
+    </row>
+    <row r="9" spans="1:2">
+      <c r="A9">
+        <v>5</v>
+      </c>
+      <c r="B9">
         <v>7</v>
       </c>
-      <c r="B8">
-        <v>3</v>
-      </c>
-      <c r="C8">
-        <v>2</v>
-      </c>
-      <c r="D8" t="s">
-        <v>25</v>
-      </c>
-      <c r="E8">
+    </row>
+    <row r="10" spans="1:2">
+      <c r="A10">
+        <v>6</v>
+      </c>
+      <c r="B10">
         <v>4</v>
       </c>
     </row>
-    <row r="9" spans="1:5">
-      <c r="A9">
-        <v>8</v>
-      </c>
-      <c r="B9">
-        <v>3</v>
-      </c>
-      <c r="C9">
-        <v>1</v>
-      </c>
-      <c r="D9" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:5">
-      <c r="A10">
-        <v>9</v>
-      </c>
-      <c r="B10">
-        <v>3</v>
-      </c>
-      <c r="C10">
-        <v>2</v>
-      </c>
-      <c r="D10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:5">
+    <row r="11" spans="1:2">
       <c r="A11">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="B11">
         <v>3</v>
       </c>
-      <c r="D11" t="s">
-        <v>31</v>
+    </row>
+    <row r="12" spans="1:2">
+      <c r="A12">
+        <v>7</v>
+      </c>
+      <c r="B12">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:2">
+      <c r="A13">
+        <v>8</v>
+      </c>
+      <c r="B13">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" spans="1:2">
+      <c r="A14">
+        <v>9</v>
+      </c>
+      <c r="B14">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="15" spans="1:2">
+      <c r="A15">
+        <v>10</v>
+      </c>
+      <c r="B15">
+        <v>8</v>
       </c>
     </row>
   </sheetData>
@@ -5806,7 +5786,7 @@
 </file>
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3992BCCC-153D-40F1-88B0-57A653F9FE93}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6411490B-BC0C-412A-8052-05A3565BEF25}">
   <dimension ref="A1:B15"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <sheetData>
@@ -5815,7 +5795,7 @@
         <v>214</v>
       </c>
       <c r="B1" t="s">
-        <v>228</v>
+        <v>234</v>
       </c>
     </row>
     <row r="2" spans="1:2">
@@ -5831,7 +5811,7 @@
         <v>2</v>
       </c>
       <c r="B3">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -5839,7 +5819,7 @@
         <v>3</v>
       </c>
       <c r="B4">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="5" spans="1:2">
@@ -5847,28 +5827,28 @@
         <v>3</v>
       </c>
       <c r="B5">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6">
+        <v>3</v>
+      </c>
+      <c r="B6">
         <v>4</v>
-      </c>
-      <c r="B6">
-        <v>5</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="B7">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="B8">
         <v>6</v>
@@ -5879,23 +5859,23 @@
         <v>5</v>
       </c>
       <c r="B9">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="B10">
-        <v>4</v>
+        <v>7</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B11">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="12" spans="1:2">
@@ -5903,7 +5883,7 @@
         <v>7</v>
       </c>
       <c r="B12">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="13" spans="1:2">
@@ -5911,7 +5891,7 @@
         <v>8</v>
       </c>
       <c r="B13">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="14" spans="1:2">
@@ -5919,7 +5899,7 @@
         <v>9</v>
       </c>
       <c r="B14">
-        <v>4</v>
+        <v>10</v>
       </c>
     </row>
     <row r="15" spans="1:2">
@@ -5927,7 +5907,7 @@
         <v>10</v>
       </c>
       <c r="B15">
-        <v>8</v>
+        <v>5</v>
       </c>
     </row>
   </sheetData>
@@ -5939,139 +5919,6 @@
 </file>
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6411490B-BC0C-412A-8052-05A3565BEF25}">
-  <dimension ref="A1:B15"/>
-  <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
-  <sheetData>
-    <row r="1" spans="1:2">
-      <c r="A1" t="s">
-        <v>214</v>
-      </c>
-      <c r="B1" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2">
-      <c r="A2">
-        <v>1</v>
-      </c>
-      <c r="B2">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:2">
-      <c r="A3">
-        <v>2</v>
-      </c>
-      <c r="B3">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:2">
-      <c r="A4">
-        <v>3</v>
-      </c>
-      <c r="B4">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="5" spans="1:2">
-      <c r="A5">
-        <v>3</v>
-      </c>
-      <c r="B5">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="6" spans="1:2">
-      <c r="A6">
-        <v>3</v>
-      </c>
-      <c r="B6">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="7" spans="1:2">
-      <c r="A7">
-        <v>3</v>
-      </c>
-      <c r="B7">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="8" spans="1:2">
-      <c r="A8">
-        <v>4</v>
-      </c>
-      <c r="B8">
-        <v>6</v>
-      </c>
-    </row>
-    <row r="9" spans="1:2">
-      <c r="A9">
-        <v>5</v>
-      </c>
-      <c r="B9">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="10" spans="1:2">
-      <c r="A10">
-        <v>5</v>
-      </c>
-      <c r="B10">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="11" spans="1:2">
-      <c r="A11">
-        <v>6</v>
-      </c>
-      <c r="B11">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="12" spans="1:2">
-      <c r="A12">
-        <v>7</v>
-      </c>
-      <c r="B12">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="13" spans="1:2">
-      <c r="A13">
-        <v>8</v>
-      </c>
-      <c r="B13">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="14" spans="1:2">
-      <c r="A14">
-        <v>9</v>
-      </c>
-      <c r="B14">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="15" spans="1:2">
-      <c r="A15">
-        <v>10</v>
-      </c>
-      <c r="B15">
-        <v>5</v>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E88F946-79CD-4577-8C70-9BE607ED0BF5}">
   <dimension ref="A1:Q124"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
@@ -6082,19 +5929,19 @@
   <sheetData>
     <row r="1" spans="1:10">
       <c r="A1" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B1" t="s">
         <v>214</v>
       </c>
       <c r="C1" t="s">
+        <v>242</v>
+      </c>
+      <c r="D1" t="s">
+        <v>243</v>
+      </c>
+      <c r="E1" t="s">
         <v>244</v>
-      </c>
-      <c r="D1" t="s">
-        <v>245</v>
-      </c>
-      <c r="E1" t="s">
-        <v>246</v>
       </c>
     </row>
     <row r="2" spans="1:10">
@@ -6104,16 +5951,16 @@
       <c r="B2">
         <v>1</v>
       </c>
-      <c r="C2" s="102">
+      <c r="C2" s="99">
         <v>45901</v>
       </c>
       <c r="D2">
         <v>0</v>
       </c>
       <c r="E2" t="s">
-        <v>248</v>
-      </c>
-      <c r="J2" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J2" s="98"/>
     </row>
     <row r="3" spans="1:10">
       <c r="A3">
@@ -6122,16 +5969,16 @@
       <c r="B3">
         <v>1</v>
       </c>
-      <c r="C3" s="102">
+      <c r="C3" s="99">
         <v>45931</v>
       </c>
       <c r="D3">
         <v>0</v>
       </c>
       <c r="E3" t="s">
-        <v>248</v>
-      </c>
-      <c r="J3" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J3" s="98"/>
     </row>
     <row r="4" spans="1:10">
       <c r="A4">
@@ -6140,16 +5987,16 @@
       <c r="B4">
         <v>1</v>
       </c>
-      <c r="C4" s="102">
+      <c r="C4" s="99">
         <v>45962</v>
       </c>
       <c r="D4">
         <v>3758</v>
       </c>
       <c r="E4" t="s">
-        <v>247</v>
-      </c>
-      <c r="J4" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J4" s="98"/>
     </row>
     <row r="5" spans="1:10">
       <c r="A5">
@@ -6158,16 +6005,16 @@
       <c r="B5">
         <v>1</v>
       </c>
-      <c r="C5" s="102">
+      <c r="C5" s="99">
         <v>45992</v>
       </c>
       <c r="D5">
         <v>0</v>
       </c>
       <c r="E5" t="s">
-        <v>248</v>
-      </c>
-      <c r="J5" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J5" s="98"/>
     </row>
     <row r="6" spans="1:10">
       <c r="A6">
@@ -6176,16 +6023,16 @@
       <c r="B6">
         <v>1</v>
       </c>
-      <c r="C6" s="102">
+      <c r="C6" s="99">
         <v>46023</v>
       </c>
       <c r="D6">
         <v>0</v>
       </c>
       <c r="E6" t="s">
-        <v>248</v>
-      </c>
-      <c r="J6" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J6" s="98"/>
     </row>
     <row r="7" spans="1:10">
       <c r="A7">
@@ -6194,16 +6041,16 @@
       <c r="B7">
         <v>1</v>
       </c>
-      <c r="C7" s="102">
+      <c r="C7" s="99">
         <v>46054</v>
       </c>
       <c r="D7">
         <v>3897</v>
       </c>
       <c r="E7" t="s">
-        <v>248</v>
-      </c>
-      <c r="J7" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J7" s="98"/>
     </row>
     <row r="8" spans="1:10">
       <c r="A8">
@@ -6212,16 +6059,16 @@
       <c r="B8">
         <v>1</v>
       </c>
-      <c r="C8" s="102">
+      <c r="C8" s="99">
         <v>46082</v>
       </c>
       <c r="D8">
         <v>5101</v>
       </c>
       <c r="E8" t="s">
-        <v>248</v>
-      </c>
-      <c r="J8" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J8" s="98"/>
     </row>
     <row r="9" spans="1:10">
       <c r="A9">
@@ -6230,16 +6077,16 @@
       <c r="B9">
         <v>1</v>
       </c>
-      <c r="C9" s="102">
+      <c r="C9" s="99">
         <v>46113</v>
       </c>
       <c r="D9">
         <v>0</v>
       </c>
       <c r="E9" t="s">
-        <v>248</v>
-      </c>
-      <c r="J9" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J9" s="98"/>
     </row>
     <row r="10" spans="1:10">
       <c r="A10">
@@ -6248,16 +6095,16 @@
       <c r="B10">
         <v>1</v>
       </c>
-      <c r="C10" s="102">
+      <c r="C10" s="99">
         <v>46143</v>
       </c>
       <c r="D10">
         <v>0</v>
       </c>
       <c r="E10" t="s">
-        <v>248</v>
-      </c>
-      <c r="J10" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J10" s="98"/>
     </row>
     <row r="11" spans="1:10">
       <c r="A11">
@@ -6266,16 +6113,16 @@
       <c r="B11">
         <v>1</v>
       </c>
-      <c r="C11" s="102">
+      <c r="C11" s="99">
         <v>46174</v>
       </c>
       <c r="D11">
         <v>0</v>
       </c>
       <c r="E11" t="s">
-        <v>248</v>
-      </c>
-      <c r="J11" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J11" s="98"/>
     </row>
     <row r="12" spans="1:10">
       <c r="A12">
@@ -6284,16 +6131,16 @@
       <c r="B12">
         <v>1</v>
       </c>
-      <c r="C12" s="102">
+      <c r="C12" s="99">
         <v>46204</v>
       </c>
       <c r="D12">
         <v>0</v>
       </c>
       <c r="E12" t="s">
-        <v>248</v>
-      </c>
-      <c r="J12" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J12" s="98"/>
     </row>
     <row r="13" spans="1:10">
       <c r="A13">
@@ -6302,16 +6149,16 @@
       <c r="B13">
         <v>1</v>
       </c>
-      <c r="C13" s="102">
+      <c r="C13" s="99">
         <v>46235</v>
       </c>
       <c r="D13">
         <v>0</v>
       </c>
       <c r="E13" t="s">
-        <v>248</v>
-      </c>
-      <c r="J13" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J13" s="98"/>
     </row>
     <row r="14" spans="1:10">
       <c r="A14">
@@ -6320,16 +6167,16 @@
       <c r="B14">
         <v>2</v>
       </c>
-      <c r="C14" s="102">
+      <c r="C14" s="99">
         <v>45901</v>
       </c>
       <c r="D14">
         <v>0</v>
       </c>
       <c r="E14" t="s">
-        <v>248</v>
-      </c>
-      <c r="J14" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J14" s="98"/>
     </row>
     <row r="15" spans="1:10">
       <c r="A15">
@@ -6338,16 +6185,16 @@
       <c r="B15">
         <v>2</v>
       </c>
-      <c r="C15" s="102">
+      <c r="C15" s="99">
         <v>45931</v>
       </c>
       <c r="D15">
         <v>0</v>
       </c>
       <c r="E15" t="s">
-        <v>248</v>
-      </c>
-      <c r="J15" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J15" s="98"/>
     </row>
     <row r="16" spans="1:10">
       <c r="A16">
@@ -6356,16 +6203,16 @@
       <c r="B16">
         <v>2</v>
       </c>
-      <c r="C16" s="102">
+      <c r="C16" s="99">
         <v>45962</v>
       </c>
       <c r="D16">
         <v>0.8327</v>
       </c>
       <c r="E16" t="s">
-        <v>247</v>
-      </c>
-      <c r="J16" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J16" s="98"/>
     </row>
     <row r="17" spans="1:15">
       <c r="A17">
@@ -6374,16 +6221,16 @@
       <c r="B17">
         <v>2</v>
       </c>
-      <c r="C17" s="102">
+      <c r="C17" s="99">
         <v>45992</v>
       </c>
       <c r="D17">
         <v>0</v>
       </c>
       <c r="E17" t="s">
-        <v>248</v>
-      </c>
-      <c r="J17" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J17" s="98"/>
     </row>
     <row r="18" spans="1:15">
       <c r="A18">
@@ -6392,16 +6239,16 @@
       <c r="B18">
         <v>2</v>
       </c>
-      <c r="C18" s="102">
+      <c r="C18" s="99">
         <v>46023</v>
       </c>
       <c r="D18">
         <v>0</v>
       </c>
       <c r="E18" t="s">
-        <v>248</v>
-      </c>
-      <c r="J18" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J18" s="98"/>
     </row>
     <row r="19" spans="1:15">
       <c r="A19">
@@ -6410,16 +6257,16 @@
       <c r="B19">
         <v>2</v>
       </c>
-      <c r="C19" s="102">
+      <c r="C19" s="99">
         <v>46054</v>
       </c>
       <c r="D19">
         <v>0.87270000000000003</v>
       </c>
       <c r="E19" t="s">
-        <v>248</v>
-      </c>
-      <c r="J19" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J19" s="98"/>
     </row>
     <row r="20" spans="1:15">
       <c r="A20">
@@ -6428,16 +6275,16 @@
       <c r="B20">
         <v>2</v>
       </c>
-      <c r="C20" s="102">
+      <c r="C20" s="99">
         <v>46082</v>
       </c>
       <c r="D20">
         <v>0</v>
       </c>
       <c r="E20" t="s">
-        <v>248</v>
-      </c>
-      <c r="J20" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J20" s="98"/>
     </row>
     <row r="21" spans="1:15">
       <c r="A21">
@@ -6446,16 +6293,16 @@
       <c r="B21">
         <v>2</v>
       </c>
-      <c r="C21" s="102">
+      <c r="C21" s="99">
         <v>46113</v>
       </c>
       <c r="D21">
         <v>0</v>
       </c>
       <c r="E21" t="s">
-        <v>248</v>
-      </c>
-      <c r="J21" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J21" s="98"/>
     </row>
     <row r="22" spans="1:15">
       <c r="A22">
@@ -6464,16 +6311,16 @@
       <c r="B22">
         <v>2</v>
       </c>
-      <c r="C22" s="102">
+      <c r="C22" s="99">
         <v>46143</v>
       </c>
       <c r="D22">
         <v>0</v>
       </c>
       <c r="E22" t="s">
-        <v>248</v>
-      </c>
-      <c r="J22" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J22" s="98"/>
     </row>
     <row r="23" spans="1:15">
       <c r="A23">
@@ -6482,16 +6329,16 @@
       <c r="B23">
         <v>2</v>
       </c>
-      <c r="C23" s="102">
+      <c r="C23" s="99">
         <v>46174</v>
       </c>
       <c r="D23">
         <v>0</v>
       </c>
       <c r="E23" t="s">
-        <v>248</v>
-      </c>
-      <c r="J23" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J23" s="98"/>
     </row>
     <row r="24" spans="1:15">
       <c r="A24">
@@ -6500,16 +6347,16 @@
       <c r="B24">
         <v>2</v>
       </c>
-      <c r="C24" s="102">
+      <c r="C24" s="99">
         <v>46204</v>
       </c>
       <c r="D24">
         <v>0</v>
       </c>
       <c r="E24" t="s">
-        <v>248</v>
-      </c>
-      <c r="J24" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J24" s="98"/>
     </row>
     <row r="25" spans="1:15">
       <c r="A25">
@@ -6518,16 +6365,16 @@
       <c r="B25">
         <v>2</v>
       </c>
-      <c r="C25" s="102">
+      <c r="C25" s="99">
         <v>46235</v>
       </c>
       <c r="D25">
         <v>0</v>
       </c>
       <c r="E25" t="s">
-        <v>248</v>
-      </c>
-      <c r="J25" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J25" s="98"/>
     </row>
     <row r="26" spans="1:15">
       <c r="A26">
@@ -6536,16 +6383,16 @@
       <c r="B26">
         <v>3</v>
       </c>
-      <c r="C26" s="102">
+      <c r="C26" s="99">
         <v>45901</v>
       </c>
       <c r="D26">
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>248</v>
-      </c>
-      <c r="J26" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J26" s="98"/>
     </row>
     <row r="27" spans="1:15">
       <c r="A27">
@@ -6554,16 +6401,16 @@
       <c r="B27">
         <v>3</v>
       </c>
-      <c r="C27" s="102">
+      <c r="C27" s="99">
         <v>45931</v>
       </c>
       <c r="D27">
         <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>248</v>
-      </c>
-      <c r="J27" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J27" s="98"/>
     </row>
     <row r="28" spans="1:15">
       <c r="A28">
@@ -6572,16 +6419,16 @@
       <c r="B28">
         <v>3</v>
       </c>
-      <c r="C28" s="102">
+      <c r="C28" s="99">
         <v>45962</v>
       </c>
       <c r="D28">
         <v>0</v>
       </c>
       <c r="E28" t="s">
-        <v>247</v>
-      </c>
-      <c r="J28" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J28" s="98"/>
     </row>
     <row r="29" spans="1:15">
       <c r="A29">
@@ -6590,16 +6437,16 @@
       <c r="B29">
         <v>3</v>
       </c>
-      <c r="C29" s="102">
+      <c r="C29" s="99">
         <v>45992</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>248</v>
-      </c>
-      <c r="J29" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J29" s="98"/>
     </row>
     <row r="30" spans="1:15">
       <c r="A30">
@@ -6608,16 +6455,16 @@
       <c r="B30">
         <v>3</v>
       </c>
-      <c r="C30" s="102">
+      <c r="C30" s="99">
         <v>46023</v>
       </c>
       <c r="D30">
         <v>2</v>
       </c>
       <c r="E30" t="s">
-        <v>248</v>
-      </c>
-      <c r="J30" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J30" s="98"/>
     </row>
     <row r="31" spans="1:15">
       <c r="A31">
@@ -6626,16 +6473,16 @@
       <c r="B31">
         <v>3</v>
       </c>
-      <c r="C31" s="102">
+      <c r="C31" s="99">
         <v>46054</v>
       </c>
       <c r="D31">
         <v>1</v>
       </c>
       <c r="E31" t="s">
-        <v>248</v>
-      </c>
-      <c r="J31" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J31" s="98"/>
       <c r="O31" s="57"/>
     </row>
     <row r="32" spans="1:15">
@@ -6645,16 +6492,16 @@
       <c r="B32">
         <v>3</v>
       </c>
-      <c r="C32" s="102">
+      <c r="C32" s="99">
         <v>46082</v>
       </c>
       <c r="D32">
         <v>0</v>
       </c>
       <c r="E32" t="s">
-        <v>248</v>
-      </c>
-      <c r="J32" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J32" s="98"/>
       <c r="O32" s="57"/>
     </row>
     <row r="33" spans="1:15">
@@ -6664,16 +6511,16 @@
       <c r="B33">
         <v>3</v>
       </c>
-      <c r="C33" s="102">
+      <c r="C33" s="99">
         <v>46113</v>
       </c>
       <c r="D33">
         <v>0</v>
       </c>
       <c r="E33" t="s">
-        <v>248</v>
-      </c>
-      <c r="J33" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J33" s="98"/>
       <c r="O33" s="57"/>
     </row>
     <row r="34" spans="1:15">
@@ -6683,16 +6530,16 @@
       <c r="B34">
         <v>3</v>
       </c>
-      <c r="C34" s="102">
+      <c r="C34" s="99">
         <v>46143</v>
       </c>
       <c r="D34">
         <v>0</v>
       </c>
       <c r="E34" t="s">
-        <v>248</v>
-      </c>
-      <c r="J34" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J34" s="98"/>
       <c r="O34" s="57"/>
     </row>
     <row r="35" spans="1:15">
@@ -6702,16 +6549,16 @@
       <c r="B35">
         <v>3</v>
       </c>
-      <c r="C35" s="102">
+      <c r="C35" s="99">
         <v>46174</v>
       </c>
       <c r="D35">
         <v>0</v>
       </c>
       <c r="E35" t="s">
-        <v>248</v>
-      </c>
-      <c r="J35" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J35" s="98"/>
       <c r="O35" s="57"/>
     </row>
     <row r="36" spans="1:15">
@@ -6721,16 +6568,16 @@
       <c r="B36">
         <v>3</v>
       </c>
-      <c r="C36" s="102">
+      <c r="C36" s="99">
         <v>46204</v>
       </c>
       <c r="D36">
         <v>0</v>
       </c>
       <c r="E36" t="s">
-        <v>248</v>
-      </c>
-      <c r="J36" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J36" s="98"/>
       <c r="O36" s="57"/>
     </row>
     <row r="37" spans="1:15">
@@ -6740,16 +6587,16 @@
       <c r="B37">
         <v>3</v>
       </c>
-      <c r="C37" s="102">
+      <c r="C37" s="99">
         <v>46235</v>
       </c>
       <c r="D37">
         <v>0</v>
       </c>
       <c r="E37" t="s">
-        <v>248</v>
-      </c>
-      <c r="J37" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J37" s="98"/>
       <c r="O37" s="57"/>
     </row>
     <row r="38" spans="1:15">
@@ -6759,16 +6606,16 @@
       <c r="B38">
         <v>4</v>
       </c>
-      <c r="C38" s="102">
+      <c r="C38" s="99">
         <v>45901</v>
       </c>
       <c r="D38">
         <v>0</v>
       </c>
       <c r="E38" t="s">
-        <v>248</v>
-      </c>
-      <c r="J38" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J38" s="98"/>
       <c r="N38" s="57"/>
       <c r="O38" s="57"/>
     </row>
@@ -6779,16 +6626,16 @@
       <c r="B39">
         <v>4</v>
       </c>
-      <c r="C39" s="102">
+      <c r="C39" s="99">
         <v>45931</v>
       </c>
       <c r="D39">
         <v>0</v>
       </c>
       <c r="E39" t="s">
-        <v>248</v>
-      </c>
-      <c r="J39" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J39" s="98"/>
       <c r="N39" s="57"/>
       <c r="O39" s="57"/>
     </row>
@@ -6799,16 +6646,16 @@
       <c r="B40">
         <v>4</v>
       </c>
-      <c r="C40" s="102">
+      <c r="C40" s="99">
         <v>45962</v>
       </c>
       <c r="D40">
         <v>0</v>
       </c>
       <c r="E40" t="s">
-        <v>247</v>
-      </c>
-      <c r="J40" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J40" s="98"/>
       <c r="N40" s="57"/>
       <c r="O40" s="57"/>
     </row>
@@ -6819,16 +6666,16 @@
       <c r="B41">
         <v>4</v>
       </c>
-      <c r="C41" s="102">
+      <c r="C41" s="99">
         <v>45992</v>
       </c>
       <c r="D41">
         <v>0</v>
       </c>
       <c r="E41" t="s">
-        <v>248</v>
-      </c>
-      <c r="J41" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J41" s="98"/>
       <c r="N41" s="57"/>
       <c r="O41" s="57"/>
     </row>
@@ -6839,16 +6686,16 @@
       <c r="B42">
         <v>4</v>
       </c>
-      <c r="C42" s="102">
+      <c r="C42" s="99">
         <v>46023</v>
       </c>
       <c r="D42">
         <v>0</v>
       </c>
       <c r="E42" t="s">
-        <v>248</v>
-      </c>
-      <c r="J42" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J42" s="98"/>
       <c r="N42" s="57"/>
       <c r="O42" s="57"/>
     </row>
@@ -6859,16 +6706,16 @@
       <c r="B43">
         <v>4</v>
       </c>
-      <c r="C43" s="102">
+      <c r="C43" s="99">
         <v>46054</v>
       </c>
       <c r="D43">
         <v>1</v>
       </c>
       <c r="E43" t="s">
-        <v>248</v>
-      </c>
-      <c r="J43" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J43" s="98"/>
       <c r="N43" s="57"/>
       <c r="O43" s="57"/>
     </row>
@@ -6879,16 +6726,16 @@
       <c r="B44">
         <v>4</v>
       </c>
-      <c r="C44" s="102">
+      <c r="C44" s="99">
         <v>46082</v>
       </c>
       <c r="D44">
         <v>0</v>
       </c>
       <c r="E44" t="s">
-        <v>248</v>
-      </c>
-      <c r="J44" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J44" s="98"/>
       <c r="N44" s="57"/>
       <c r="O44" s="57"/>
     </row>
@@ -6899,16 +6746,16 @@
       <c r="B45">
         <v>4</v>
       </c>
-      <c r="C45" s="102">
+      <c r="C45" s="99">
         <v>46113</v>
       </c>
       <c r="D45">
         <v>0</v>
       </c>
       <c r="E45" t="s">
-        <v>248</v>
-      </c>
-      <c r="J45" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J45" s="98"/>
       <c r="N45" s="57"/>
       <c r="O45" s="57"/>
     </row>
@@ -6919,16 +6766,16 @@
       <c r="B46">
         <v>4</v>
       </c>
-      <c r="C46" s="102">
+      <c r="C46" s="99">
         <v>46143</v>
       </c>
       <c r="D46">
         <v>0</v>
       </c>
       <c r="E46" t="s">
-        <v>248</v>
-      </c>
-      <c r="J46" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J46" s="98"/>
       <c r="N46" s="57"/>
       <c r="O46" s="57"/>
     </row>
@@ -6939,16 +6786,16 @@
       <c r="B47">
         <v>4</v>
       </c>
-      <c r="C47" s="102">
+      <c r="C47" s="99">
         <v>46174</v>
       </c>
       <c r="D47">
         <v>0</v>
       </c>
       <c r="E47" t="s">
-        <v>248</v>
-      </c>
-      <c r="J47" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J47" s="98"/>
       <c r="N47" s="57"/>
       <c r="O47" s="57"/>
     </row>
@@ -6959,16 +6806,16 @@
       <c r="B48">
         <v>4</v>
       </c>
-      <c r="C48" s="102">
+      <c r="C48" s="99">
         <v>46204</v>
       </c>
       <c r="D48">
         <v>0</v>
       </c>
       <c r="E48" t="s">
-        <v>248</v>
-      </c>
-      <c r="J48" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J48" s="98"/>
       <c r="N48" s="57"/>
       <c r="O48" s="57"/>
     </row>
@@ -6979,16 +6826,16 @@
       <c r="B49">
         <v>4</v>
       </c>
-      <c r="C49" s="102">
+      <c r="C49" s="99">
         <v>46235</v>
       </c>
       <c r="D49">
         <v>0</v>
       </c>
       <c r="E49" t="s">
-        <v>248</v>
-      </c>
-      <c r="J49" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J49" s="98"/>
       <c r="L49" s="57"/>
       <c r="N49" s="57"/>
       <c r="O49" s="57"/>
@@ -7000,16 +6847,16 @@
       <c r="B50">
         <v>5</v>
       </c>
-      <c r="C50" s="102">
+      <c r="C50" s="99">
         <v>45901</v>
       </c>
       <c r="D50">
         <v>13</v>
       </c>
       <c r="E50" t="s">
-        <v>248</v>
-      </c>
-      <c r="J50" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J50" s="98"/>
       <c r="L50" s="57"/>
       <c r="O50" s="57"/>
     </row>
@@ -7020,16 +6867,16 @@
       <c r="B51">
         <v>5</v>
       </c>
-      <c r="C51" s="102">
+      <c r="C51" s="99">
         <v>45931</v>
       </c>
       <c r="D51">
         <v>18</v>
       </c>
       <c r="E51" t="s">
-        <v>248</v>
-      </c>
-      <c r="J51" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J51" s="98"/>
       <c r="L51" s="57"/>
       <c r="O51" s="57"/>
     </row>
@@ -7040,16 +6887,16 @@
       <c r="B52">
         <v>5</v>
       </c>
-      <c r="C52" s="102">
+      <c r="C52" s="99">
         <v>45962</v>
       </c>
       <c r="D52">
         <v>9</v>
       </c>
       <c r="E52" t="s">
-        <v>247</v>
-      </c>
-      <c r="J52" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J52" s="98"/>
       <c r="L52" s="57"/>
       <c r="O52" s="57"/>
     </row>
@@ -7060,16 +6907,16 @@
       <c r="B53">
         <v>5</v>
       </c>
-      <c r="C53" s="102">
+      <c r="C53" s="99">
         <v>45992</v>
       </c>
       <c r="D53">
         <v>7</v>
       </c>
       <c r="E53" t="s">
-        <v>248</v>
-      </c>
-      <c r="J53" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J53" s="98"/>
       <c r="L53" s="57"/>
       <c r="O53" s="57"/>
     </row>
@@ -7080,16 +6927,16 @@
       <c r="B54">
         <v>5</v>
       </c>
-      <c r="C54" s="102">
+      <c r="C54" s="99">
         <v>46023</v>
       </c>
       <c r="D54">
         <v>7</v>
       </c>
       <c r="E54" t="s">
-        <v>248</v>
-      </c>
-      <c r="J54" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J54" s="98"/>
       <c r="L54" s="57"/>
     </row>
     <row r="55" spans="1:17">
@@ -7099,16 +6946,16 @@
       <c r="B55">
         <v>5</v>
       </c>
-      <c r="C55" s="102">
+      <c r="C55" s="99">
         <v>46054</v>
       </c>
       <c r="D55">
         <v>7</v>
       </c>
       <c r="E55" t="s">
-        <v>248</v>
-      </c>
-      <c r="J55" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J55" s="98"/>
       <c r="L55" s="57"/>
     </row>
     <row r="56" spans="1:17">
@@ -7118,16 +6965,16 @@
       <c r="B56">
         <v>5</v>
       </c>
-      <c r="C56" s="102">
+      <c r="C56" s="99">
         <v>46082</v>
       </c>
       <c r="D56">
         <v>0</v>
       </c>
       <c r="E56" t="s">
-        <v>248</v>
-      </c>
-      <c r="J56" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J56" s="98"/>
       <c r="L56" s="57"/>
     </row>
     <row r="57" spans="1:17">
@@ -7137,16 +6984,16 @@
       <c r="B57">
         <v>5</v>
       </c>
-      <c r="C57" s="102">
+      <c r="C57" s="99">
         <v>46113</v>
       </c>
       <c r="D57">
         <v>0</v>
       </c>
       <c r="E57" t="s">
-        <v>248</v>
-      </c>
-      <c r="J57" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J57" s="98"/>
       <c r="L57" s="57"/>
     </row>
     <row r="58" spans="1:17">
@@ -7156,16 +7003,16 @@
       <c r="B58">
         <v>5</v>
       </c>
-      <c r="C58" s="102">
+      <c r="C58" s="99">
         <v>46143</v>
       </c>
       <c r="D58">
         <v>0</v>
       </c>
       <c r="E58" t="s">
-        <v>248</v>
-      </c>
-      <c r="J58" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J58" s="98"/>
       <c r="L58" s="57"/>
     </row>
     <row r="59" spans="1:17">
@@ -7175,16 +7022,16 @@
       <c r="B59">
         <v>5</v>
       </c>
-      <c r="C59" s="102">
+      <c r="C59" s="99">
         <v>46174</v>
       </c>
       <c r="D59">
         <v>0</v>
       </c>
       <c r="E59" t="s">
-        <v>248</v>
-      </c>
-      <c r="J59" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J59" s="98"/>
       <c r="L59" s="57"/>
     </row>
     <row r="60" spans="1:17">
@@ -7194,16 +7041,16 @@
       <c r="B60">
         <v>5</v>
       </c>
-      <c r="C60" s="102">
+      <c r="C60" s="99">
         <v>46204</v>
       </c>
       <c r="D60">
         <v>0</v>
       </c>
       <c r="E60" t="s">
-        <v>248</v>
-      </c>
-      <c r="J60" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J60" s="98"/>
       <c r="L60" s="57"/>
     </row>
     <row r="61" spans="1:17">
@@ -7213,16 +7060,16 @@
       <c r="B61">
         <v>5</v>
       </c>
-      <c r="C61" s="102">
+      <c r="C61" s="99">
         <v>46235</v>
       </c>
       <c r="D61">
         <v>0</v>
       </c>
       <c r="E61" t="s">
-        <v>248</v>
-      </c>
-      <c r="J61" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J61" s="98"/>
     </row>
     <row r="62" spans="1:17">
       <c r="A62">
@@ -7231,16 +7078,16 @@
       <c r="B62">
         <v>6</v>
       </c>
-      <c r="C62" s="102">
+      <c r="C62" s="99">
         <v>45901</v>
       </c>
       <c r="D62">
         <v>0</v>
       </c>
       <c r="E62" t="s">
-        <v>248</v>
-      </c>
-      <c r="J62" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J62" s="98"/>
     </row>
     <row r="63" spans="1:17">
       <c r="A63">
@@ -7249,16 +7096,16 @@
       <c r="B63">
         <v>6</v>
       </c>
-      <c r="C63" s="102">
+      <c r="C63" s="99">
         <v>45931</v>
       </c>
       <c r="D63">
         <v>0</v>
       </c>
       <c r="E63" t="s">
-        <v>248</v>
-      </c>
-      <c r="J63" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J63" s="98"/>
       <c r="Q63" s="57"/>
     </row>
     <row r="64" spans="1:17">
@@ -7268,16 +7115,16 @@
       <c r="B64">
         <v>6</v>
       </c>
-      <c r="C64" s="102">
+      <c r="C64" s="99">
         <v>45962</v>
       </c>
       <c r="D64">
         <v>1</v>
       </c>
       <c r="E64" t="s">
-        <v>247</v>
-      </c>
-      <c r="J64" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J64" s="98"/>
       <c r="Q64" s="57"/>
     </row>
     <row r="65" spans="1:17">
@@ -7287,16 +7134,16 @@
       <c r="B65">
         <v>6</v>
       </c>
-      <c r="C65" s="102">
+      <c r="C65" s="99">
         <v>45992</v>
       </c>
       <c r="D65">
         <v>1</v>
       </c>
       <c r="E65" t="s">
-        <v>248</v>
-      </c>
-      <c r="J65" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J65" s="98"/>
       <c r="Q65" s="57"/>
     </row>
     <row r="66" spans="1:17">
@@ -7306,16 +7153,16 @@
       <c r="B66">
         <v>6</v>
       </c>
-      <c r="C66" s="102">
+      <c r="C66" s="99">
         <v>46023</v>
       </c>
       <c r="D66">
         <v>1</v>
       </c>
       <c r="E66" t="s">
-        <v>248</v>
-      </c>
-      <c r="J66" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J66" s="98"/>
       <c r="Q66" s="57"/>
     </row>
     <row r="67" spans="1:17">
@@ -7325,16 +7172,16 @@
       <c r="B67">
         <v>6</v>
       </c>
-      <c r="C67" s="102">
+      <c r="C67" s="99">
         <v>46054</v>
       </c>
       <c r="D67">
         <v>1</v>
       </c>
       <c r="E67" t="s">
-        <v>248</v>
-      </c>
-      <c r="J67" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J67" s="98"/>
       <c r="Q67" s="57"/>
     </row>
     <row r="68" spans="1:17">
@@ -7344,16 +7191,16 @@
       <c r="B68">
         <v>6</v>
       </c>
-      <c r="C68" s="102">
+      <c r="C68" s="99">
         <v>46082</v>
       </c>
       <c r="D68">
         <v>0</v>
       </c>
       <c r="E68" t="s">
-        <v>248</v>
-      </c>
-      <c r="J68" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J68" s="98"/>
       <c r="Q68" s="57"/>
     </row>
     <row r="69" spans="1:17">
@@ -7363,16 +7210,16 @@
       <c r="B69">
         <v>6</v>
       </c>
-      <c r="C69" s="102">
+      <c r="C69" s="99">
         <v>46113</v>
       </c>
       <c r="D69">
         <v>0</v>
       </c>
       <c r="E69" t="s">
-        <v>248</v>
-      </c>
-      <c r="J69" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J69" s="98"/>
       <c r="Q69" s="57"/>
     </row>
     <row r="70" spans="1:17">
@@ -7382,16 +7229,16 @@
       <c r="B70">
         <v>6</v>
       </c>
-      <c r="C70" s="102">
+      <c r="C70" s="99">
         <v>46143</v>
       </c>
       <c r="D70">
         <v>0</v>
       </c>
       <c r="E70" t="s">
-        <v>248</v>
-      </c>
-      <c r="J70" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J70" s="98"/>
       <c r="Q70" s="57"/>
     </row>
     <row r="71" spans="1:17">
@@ -7401,16 +7248,16 @@
       <c r="B71">
         <v>6</v>
       </c>
-      <c r="C71" s="102">
+      <c r="C71" s="99">
         <v>46174</v>
       </c>
       <c r="D71">
         <v>0</v>
       </c>
       <c r="E71" t="s">
-        <v>248</v>
-      </c>
-      <c r="J71" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J71" s="98"/>
       <c r="Q71" s="57"/>
     </row>
     <row r="72" spans="1:17">
@@ -7420,16 +7267,16 @@
       <c r="B72">
         <v>6</v>
       </c>
-      <c r="C72" s="102">
+      <c r="C72" s="99">
         <v>46204</v>
       </c>
       <c r="D72">
         <v>0</v>
       </c>
       <c r="E72" t="s">
-        <v>248</v>
-      </c>
-      <c r="J72" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J72" s="98"/>
       <c r="Q72" s="57"/>
     </row>
     <row r="73" spans="1:17">
@@ -7439,16 +7286,16 @@
       <c r="B73">
         <v>6</v>
       </c>
-      <c r="C73" s="102">
+      <c r="C73" s="99">
         <v>46235</v>
       </c>
       <c r="D73">
         <v>0</v>
       </c>
       <c r="E73" t="s">
-        <v>248</v>
-      </c>
-      <c r="J73" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J73" s="98"/>
       <c r="Q73" s="57"/>
     </row>
     <row r="74" spans="1:17">
@@ -7458,16 +7305,16 @@
       <c r="B74">
         <v>7</v>
       </c>
-      <c r="C74" s="102">
+      <c r="C74" s="99">
         <v>45901</v>
       </c>
       <c r="D74">
         <v>0</v>
       </c>
       <c r="E74" t="s">
-        <v>248</v>
-      </c>
-      <c r="J74" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J74" s="98"/>
       <c r="Q74" s="57"/>
     </row>
     <row r="75" spans="1:17">
@@ -7477,16 +7324,16 @@
       <c r="B75">
         <v>7</v>
       </c>
-      <c r="C75" s="102">
+      <c r="C75" s="99">
         <v>45931</v>
       </c>
       <c r="D75">
         <v>0</v>
       </c>
       <c r="E75" t="s">
-        <v>248</v>
-      </c>
-      <c r="J75" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J75" s="98"/>
     </row>
     <row r="76" spans="1:17">
       <c r="A76">
@@ -7495,16 +7342,16 @@
       <c r="B76">
         <v>7</v>
       </c>
-      <c r="C76" s="102">
+      <c r="C76" s="99">
         <v>45962</v>
       </c>
       <c r="D76">
         <v>0</v>
       </c>
       <c r="E76" t="s">
-        <v>247</v>
-      </c>
-      <c r="J76" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J76" s="98"/>
     </row>
     <row r="77" spans="1:17">
       <c r="A77">
@@ -7513,16 +7360,16 @@
       <c r="B77">
         <v>7</v>
       </c>
-      <c r="C77" s="102">
+      <c r="C77" s="99">
         <v>45992</v>
       </c>
       <c r="D77">
         <v>0</v>
       </c>
       <c r="E77" t="s">
-        <v>248</v>
-      </c>
-      <c r="J77" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J77" s="98"/>
     </row>
     <row r="78" spans="1:17">
       <c r="A78">
@@ -7531,16 +7378,16 @@
       <c r="B78">
         <v>7</v>
       </c>
-      <c r="C78" s="102">
+      <c r="C78" s="99">
         <v>46023</v>
       </c>
       <c r="D78">
         <v>0</v>
       </c>
       <c r="E78" t="s">
-        <v>248</v>
-      </c>
-      <c r="J78" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J78" s="98"/>
     </row>
     <row r="79" spans="1:17">
       <c r="A79">
@@ -7549,16 +7396,16 @@
       <c r="B79">
         <v>7</v>
       </c>
-      <c r="C79" s="102">
+      <c r="C79" s="99">
         <v>46054</v>
       </c>
       <c r="D79">
         <v>1</v>
       </c>
       <c r="E79" t="s">
-        <v>248</v>
-      </c>
-      <c r="J79" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J79" s="98"/>
     </row>
     <row r="80" spans="1:17">
       <c r="A80">
@@ -7567,16 +7414,16 @@
       <c r="B80">
         <v>7</v>
       </c>
-      <c r="C80" s="102">
+      <c r="C80" s="99">
         <v>46082</v>
       </c>
       <c r="D80">
         <v>0</v>
       </c>
       <c r="E80" t="s">
-        <v>248</v>
-      </c>
-      <c r="J80" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J80" s="98"/>
     </row>
     <row r="81" spans="1:15">
       <c r="A81">
@@ -7585,16 +7432,16 @@
       <c r="B81">
         <v>7</v>
       </c>
-      <c r="C81" s="102">
+      <c r="C81" s="99">
         <v>46113</v>
       </c>
       <c r="D81">
         <v>0</v>
       </c>
       <c r="E81" t="s">
-        <v>248</v>
-      </c>
-      <c r="J81" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J81" s="98"/>
       <c r="K81" s="57"/>
     </row>
     <row r="82" spans="1:15">
@@ -7604,16 +7451,16 @@
       <c r="B82">
         <v>7</v>
       </c>
-      <c r="C82" s="102">
+      <c r="C82" s="99">
         <v>46143</v>
       </c>
       <c r="D82">
         <v>0</v>
       </c>
       <c r="E82" t="s">
-        <v>248</v>
-      </c>
-      <c r="J82" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J82" s="98"/>
       <c r="K82" s="57"/>
     </row>
     <row r="83" spans="1:15">
@@ -7623,16 +7470,16 @@
       <c r="B83">
         <v>7</v>
       </c>
-      <c r="C83" s="102">
+      <c r="C83" s="99">
         <v>46174</v>
       </c>
       <c r="D83">
         <v>0</v>
       </c>
       <c r="E83" t="s">
-        <v>248</v>
-      </c>
-      <c r="J83" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J83" s="98"/>
       <c r="K83" s="57"/>
     </row>
     <row r="84" spans="1:15">
@@ -7642,16 +7489,16 @@
       <c r="B84">
         <v>7</v>
       </c>
-      <c r="C84" s="102">
+      <c r="C84" s="99">
         <v>46204</v>
       </c>
       <c r="D84">
         <v>0</v>
       </c>
       <c r="E84" t="s">
-        <v>248</v>
-      </c>
-      <c r="J84" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J84" s="98"/>
       <c r="K84" s="57"/>
     </row>
     <row r="85" spans="1:15">
@@ -7661,16 +7508,16 @@
       <c r="B85">
         <v>7</v>
       </c>
-      <c r="C85" s="102">
+      <c r="C85" s="99">
         <v>46235</v>
       </c>
       <c r="D85">
         <v>0</v>
       </c>
       <c r="E85" t="s">
-        <v>248</v>
-      </c>
-      <c r="J85" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J85" s="98"/>
       <c r="K85" s="57"/>
     </row>
     <row r="86" spans="1:15">
@@ -7680,16 +7527,16 @@
       <c r="B86">
         <v>8</v>
       </c>
-      <c r="C86" s="102">
+      <c r="C86" s="99">
         <v>45901</v>
       </c>
       <c r="D86">
         <v>0.8</v>
       </c>
       <c r="E86" t="s">
-        <v>248</v>
-      </c>
-      <c r="J86" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J86" s="98"/>
       <c r="K86" s="57"/>
     </row>
     <row r="87" spans="1:15">
@@ -7699,16 +7546,16 @@
       <c r="B87">
         <v>8</v>
       </c>
-      <c r="C87" s="102">
+      <c r="C87" s="99">
         <v>45931</v>
       </c>
       <c r="D87">
         <v>0.8</v>
       </c>
       <c r="E87" t="s">
-        <v>248</v>
-      </c>
-      <c r="J87" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J87" s="98"/>
       <c r="K87" s="57"/>
     </row>
     <row r="88" spans="1:15">
@@ -7718,16 +7565,16 @@
       <c r="B88">
         <v>8</v>
       </c>
-      <c r="C88" s="102">
+      <c r="C88" s="99">
         <v>45962</v>
       </c>
       <c r="D88">
         <v>0.8</v>
       </c>
       <c r="E88" t="s">
-        <v>247</v>
-      </c>
-      <c r="J88" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J88" s="98"/>
       <c r="K88" s="57"/>
     </row>
     <row r="89" spans="1:15">
@@ -7737,16 +7584,16 @@
       <c r="B89">
         <v>8</v>
       </c>
-      <c r="C89" s="102">
+      <c r="C89" s="99">
         <v>45992</v>
       </c>
       <c r="D89">
         <v>0.8</v>
       </c>
       <c r="E89" t="s">
-        <v>248</v>
-      </c>
-      <c r="J89" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J89" s="98"/>
       <c r="K89" s="57"/>
     </row>
     <row r="90" spans="1:15">
@@ -7756,16 +7603,16 @@
       <c r="B90">
         <v>8</v>
       </c>
-      <c r="C90" s="102">
+      <c r="C90" s="99">
         <v>46023</v>
       </c>
       <c r="D90">
         <v>0.8</v>
       </c>
       <c r="E90" t="s">
-        <v>248</v>
-      </c>
-      <c r="J90" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J90" s="98"/>
       <c r="K90" s="57"/>
     </row>
     <row r="91" spans="1:15">
@@ -7775,16 +7622,16 @@
       <c r="B91">
         <v>8</v>
       </c>
-      <c r="C91" s="102">
+      <c r="C91" s="99">
         <v>46054</v>
       </c>
       <c r="D91">
         <v>0.8</v>
       </c>
       <c r="E91" t="s">
-        <v>248</v>
-      </c>
-      <c r="J91" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J91" s="98"/>
       <c r="K91" s="57"/>
       <c r="N91" s="57"/>
       <c r="O91" s="1"/>
@@ -7796,16 +7643,16 @@
       <c r="B92">
         <v>8</v>
       </c>
-      <c r="C92" s="102">
+      <c r="C92" s="99">
         <v>46082</v>
       </c>
       <c r="D92">
         <v>1</v>
       </c>
       <c r="E92" t="s">
-        <v>248</v>
-      </c>
-      <c r="J92" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J92" s="98"/>
       <c r="K92" s="57"/>
       <c r="N92" s="57"/>
       <c r="O92" s="1"/>
@@ -7817,16 +7664,16 @@
       <c r="B93">
         <v>8</v>
       </c>
-      <c r="C93" s="102">
+      <c r="C93" s="99">
         <v>46113</v>
       </c>
       <c r="D93">
         <v>0</v>
       </c>
       <c r="E93" t="s">
-        <v>248</v>
-      </c>
-      <c r="J93" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J93" s="98"/>
       <c r="N93" s="57"/>
       <c r="O93" s="1"/>
     </row>
@@ -7837,16 +7684,16 @@
       <c r="B94">
         <v>8</v>
       </c>
-      <c r="C94" s="102">
+      <c r="C94" s="99">
         <v>46143</v>
       </c>
       <c r="D94">
         <v>0</v>
       </c>
       <c r="E94" t="s">
-        <v>248</v>
-      </c>
-      <c r="J94" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J94" s="98"/>
       <c r="N94" s="57"/>
       <c r="O94" s="1"/>
     </row>
@@ -7857,16 +7704,16 @@
       <c r="B95">
         <v>8</v>
       </c>
-      <c r="C95" s="102">
+      <c r="C95" s="99">
         <v>46174</v>
       </c>
       <c r="D95">
         <v>0</v>
       </c>
       <c r="E95" t="s">
-        <v>248</v>
-      </c>
-      <c r="J95" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J95" s="98"/>
       <c r="N95" s="57"/>
       <c r="O95" s="1"/>
     </row>
@@ -7877,16 +7724,16 @@
       <c r="B96">
         <v>8</v>
       </c>
-      <c r="C96" s="102">
+      <c r="C96" s="99">
         <v>46204</v>
       </c>
       <c r="D96">
         <v>0</v>
       </c>
       <c r="E96" t="s">
-        <v>248</v>
-      </c>
-      <c r="J96" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J96" s="98"/>
       <c r="N96" s="57"/>
       <c r="O96" s="1"/>
     </row>
@@ -7897,16 +7744,16 @@
       <c r="B97">
         <v>8</v>
       </c>
-      <c r="C97" s="102">
+      <c r="C97" s="99">
         <v>46235</v>
       </c>
       <c r="D97">
         <v>0</v>
       </c>
       <c r="E97" t="s">
-        <v>248</v>
-      </c>
-      <c r="J97" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J97" s="98"/>
       <c r="N97" s="57"/>
       <c r="O97" s="1"/>
     </row>
@@ -7917,16 +7764,16 @@
       <c r="B98">
         <v>9</v>
       </c>
-      <c r="C98" s="102">
+      <c r="C98" s="99">
         <v>45901</v>
       </c>
       <c r="D98">
         <v>0</v>
       </c>
       <c r="E98" t="s">
-        <v>248</v>
-      </c>
-      <c r="J98" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J98" s="98"/>
       <c r="N98" s="57"/>
       <c r="O98" s="1"/>
     </row>
@@ -7937,16 +7784,16 @@
       <c r="B99">
         <v>9</v>
       </c>
-      <c r="C99" s="102">
+      <c r="C99" s="99">
         <v>45931</v>
       </c>
       <c r="D99">
         <v>0</v>
       </c>
       <c r="E99" t="s">
-        <v>248</v>
-      </c>
-      <c r="J99" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J99" s="98"/>
       <c r="N99" s="57"/>
     </row>
     <row r="100" spans="1:15">
@@ -7956,16 +7803,16 @@
       <c r="B100">
         <v>9</v>
       </c>
-      <c r="C100" s="102">
+      <c r="C100" s="99">
         <v>45962</v>
       </c>
       <c r="D100">
         <v>0</v>
       </c>
       <c r="E100" t="s">
-        <v>247</v>
-      </c>
-      <c r="J100" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J100" s="98"/>
       <c r="N100" s="57"/>
     </row>
     <row r="101" spans="1:15">
@@ -7975,16 +7822,16 @@
       <c r="B101">
         <v>9</v>
       </c>
-      <c r="C101" s="102">
+      <c r="C101" s="99">
         <v>45992</v>
       </c>
       <c r="D101">
         <v>1</v>
       </c>
       <c r="E101" t="s">
-        <v>248</v>
-      </c>
-      <c r="J101" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J101" s="98"/>
       <c r="N101" s="57"/>
     </row>
     <row r="102" spans="1:15">
@@ -7994,16 +7841,16 @@
       <c r="B102">
         <v>9</v>
       </c>
-      <c r="C102" s="102">
+      <c r="C102" s="99">
         <v>46023</v>
       </c>
       <c r="D102">
         <v>0</v>
       </c>
       <c r="E102" t="s">
-        <v>248</v>
-      </c>
-      <c r="J102" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J102" s="98"/>
       <c r="N102" s="57"/>
     </row>
     <row r="103" spans="1:15">
@@ -8013,16 +7860,16 @@
       <c r="B103">
         <v>9</v>
       </c>
-      <c r="C103" s="102">
+      <c r="C103" s="99">
         <v>46054</v>
       </c>
       <c r="D103">
         <v>0</v>
       </c>
       <c r="E103" t="s">
-        <v>248</v>
-      </c>
-      <c r="J103" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J103" s="98"/>
     </row>
     <row r="104" spans="1:15">
       <c r="A104">
@@ -8031,16 +7878,16 @@
       <c r="B104">
         <v>9</v>
       </c>
-      <c r="C104" s="102">
+      <c r="C104" s="99">
         <v>46082</v>
       </c>
       <c r="D104">
         <v>0</v>
       </c>
       <c r="E104" t="s">
-        <v>248</v>
-      </c>
-      <c r="J104" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J104" s="98"/>
     </row>
     <row r="105" spans="1:15">
       <c r="A105">
@@ -8049,16 +7896,16 @@
       <c r="B105">
         <v>9</v>
       </c>
-      <c r="C105" s="102">
+      <c r="C105" s="99">
         <v>46113</v>
       </c>
       <c r="D105">
         <v>0</v>
       </c>
       <c r="E105" t="s">
-        <v>248</v>
-      </c>
-      <c r="J105" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J105" s="98"/>
     </row>
     <row r="106" spans="1:15">
       <c r="A106">
@@ -8067,16 +7914,16 @@
       <c r="B106">
         <v>9</v>
       </c>
-      <c r="C106" s="102">
+      <c r="C106" s="99">
         <v>46143</v>
       </c>
       <c r="D106">
         <v>0</v>
       </c>
       <c r="E106" t="s">
-        <v>248</v>
-      </c>
-      <c r="J106" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J106" s="98"/>
     </row>
     <row r="107" spans="1:15">
       <c r="A107">
@@ -8085,16 +7932,16 @@
       <c r="B107">
         <v>9</v>
       </c>
-      <c r="C107" s="102">
+      <c r="C107" s="99">
         <v>46174</v>
       </c>
       <c r="D107">
         <v>0</v>
       </c>
       <c r="E107" t="s">
-        <v>248</v>
-      </c>
-      <c r="J107" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J107" s="98"/>
     </row>
     <row r="108" spans="1:15">
       <c r="A108">
@@ -8103,16 +7950,16 @@
       <c r="B108">
         <v>9</v>
       </c>
-      <c r="C108" s="102">
+      <c r="C108" s="99">
         <v>46204</v>
       </c>
       <c r="D108">
         <v>0</v>
       </c>
       <c r="E108" t="s">
-        <v>248</v>
-      </c>
-      <c r="J108" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J108" s="98"/>
     </row>
     <row r="109" spans="1:15">
       <c r="A109">
@@ -8121,16 +7968,16 @@
       <c r="B109">
         <v>9</v>
       </c>
-      <c r="C109" s="102">
+      <c r="C109" s="99">
         <v>46235</v>
       </c>
       <c r="D109">
         <v>0</v>
       </c>
       <c r="E109" t="s">
-        <v>248</v>
-      </c>
-      <c r="J109" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J109" s="98"/>
     </row>
     <row r="110" spans="1:15">
       <c r="A110">
@@ -8139,16 +7986,16 @@
       <c r="B110">
         <v>10</v>
       </c>
-      <c r="C110" s="102">
+      <c r="C110" s="99">
         <v>45901</v>
       </c>
       <c r="D110">
         <v>0</v>
       </c>
       <c r="E110" t="s">
-        <v>248</v>
-      </c>
-      <c r="J110" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J110" s="98"/>
     </row>
     <row r="111" spans="1:15">
       <c r="A111">
@@ -8157,16 +8004,16 @@
       <c r="B111">
         <v>10</v>
       </c>
-      <c r="C111" s="102">
+      <c r="C111" s="99">
         <v>45931</v>
       </c>
       <c r="D111">
         <v>0</v>
       </c>
       <c r="E111" t="s">
-        <v>248</v>
-      </c>
-      <c r="J111" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J111" s="98"/>
     </row>
     <row r="112" spans="1:15">
       <c r="A112">
@@ -8175,16 +8022,16 @@
       <c r="B112">
         <v>10</v>
       </c>
-      <c r="C112" s="102">
+      <c r="C112" s="99">
         <v>45962</v>
       </c>
       <c r="D112">
         <v>0</v>
       </c>
       <c r="E112" t="s">
-        <v>247</v>
-      </c>
-      <c r="J112" s="101"/>
+        <v>245</v>
+      </c>
+      <c r="J112" s="98"/>
     </row>
     <row r="113" spans="1:11">
       <c r="A113">
@@ -8193,16 +8040,16 @@
       <c r="B113">
         <v>10</v>
       </c>
-      <c r="C113" s="102">
+      <c r="C113" s="99">
         <v>45992</v>
       </c>
       <c r="D113">
         <v>0</v>
       </c>
       <c r="E113" t="s">
-        <v>248</v>
-      </c>
-      <c r="J113" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J113" s="98"/>
       <c r="K113" s="57"/>
     </row>
     <row r="114" spans="1:11">
@@ -8212,16 +8059,16 @@
       <c r="B114">
         <v>10</v>
       </c>
-      <c r="C114" s="102">
+      <c r="C114" s="99">
         <v>46023</v>
       </c>
       <c r="D114">
         <v>0</v>
       </c>
       <c r="E114" t="s">
-        <v>248</v>
-      </c>
-      <c r="J114" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J114" s="98"/>
       <c r="K114" s="57"/>
     </row>
     <row r="115" spans="1:11">
@@ -8231,16 +8078,16 @@
       <c r="B115">
         <v>10</v>
       </c>
-      <c r="C115" s="102">
+      <c r="C115" s="99">
         <v>46054</v>
       </c>
       <c r="D115">
         <v>0</v>
       </c>
       <c r="E115" t="s">
-        <v>248</v>
-      </c>
-      <c r="J115" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J115" s="98"/>
       <c r="K115" s="57"/>
     </row>
     <row r="116" spans="1:11">
@@ -8250,16 +8097,16 @@
       <c r="B116">
         <v>10</v>
       </c>
-      <c r="C116" s="102">
+      <c r="C116" s="99">
         <v>46082</v>
       </c>
       <c r="D116">
         <v>0</v>
       </c>
       <c r="E116" t="s">
-        <v>248</v>
-      </c>
-      <c r="J116" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J116" s="98"/>
       <c r="K116" s="57"/>
     </row>
     <row r="117" spans="1:11">
@@ -8269,16 +8116,16 @@
       <c r="B117">
         <v>10</v>
       </c>
-      <c r="C117" s="102">
+      <c r="C117" s="99">
         <v>46113</v>
       </c>
       <c r="D117">
         <v>0</v>
       </c>
       <c r="E117" t="s">
-        <v>248</v>
-      </c>
-      <c r="J117" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J117" s="98"/>
       <c r="K117" s="57"/>
     </row>
     <row r="118" spans="1:11">
@@ -8288,16 +8135,16 @@
       <c r="B118">
         <v>10</v>
       </c>
-      <c r="C118" s="102">
+      <c r="C118" s="99">
         <v>46143</v>
       </c>
       <c r="D118">
         <v>0</v>
       </c>
       <c r="E118" t="s">
-        <v>248</v>
-      </c>
-      <c r="J118" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J118" s="98"/>
       <c r="K118" s="57"/>
     </row>
     <row r="119" spans="1:11">
@@ -8307,16 +8154,16 @@
       <c r="B119">
         <v>10</v>
       </c>
-      <c r="C119" s="102">
+      <c r="C119" s="99">
         <v>46174</v>
       </c>
       <c r="D119">
         <v>0</v>
       </c>
       <c r="E119" t="s">
-        <v>248</v>
-      </c>
-      <c r="J119" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J119" s="98"/>
       <c r="K119" s="57"/>
     </row>
     <row r="120" spans="1:11">
@@ -8326,16 +8173,16 @@
       <c r="B120">
         <v>10</v>
       </c>
-      <c r="C120" s="102">
+      <c r="C120" s="99">
         <v>46204</v>
       </c>
       <c r="D120">
         <v>0</v>
       </c>
       <c r="E120" t="s">
-        <v>248</v>
-      </c>
-      <c r="J120" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J120" s="98"/>
       <c r="K120" s="57"/>
     </row>
     <row r="121" spans="1:11">
@@ -8345,16 +8192,16 @@
       <c r="B121">
         <v>10</v>
       </c>
-      <c r="C121" s="102">
+      <c r="C121" s="99">
         <v>46235</v>
       </c>
       <c r="D121">
         <v>0</v>
       </c>
       <c r="E121" t="s">
-        <v>248</v>
-      </c>
-      <c r="J121" s="101"/>
+        <v>246</v>
+      </c>
+      <c r="J121" s="98"/>
       <c r="K121" s="57"/>
     </row>
     <row r="122" spans="1:11">
@@ -8374,7 +8221,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{B2C43C22-3382-D94C-AF1F-BAB48F8FB89E}">
   <dimension ref="A1:X33"/>
   <sheetFormatPr defaultColWidth="11" defaultRowHeight="15.75" customHeight="1"/>
@@ -8412,7 +8259,7 @@
         <v>5</v>
       </c>
       <c r="G1" s="47" t="s">
-        <v>249</v>
+        <v>247</v>
       </c>
       <c r="H1" s="47" t="s">
         <v>44</v>
@@ -8481,12 +8328,12 @@
         <v>0.2</v>
       </c>
       <c r="F2" s="60">
-        <v>986</v>
+        <v>3758</v>
       </c>
       <c r="G2" s="41"/>
       <c r="H2" s="41"/>
       <c r="I2" s="41">
-        <v>986</v>
+        <v>3758</v>
       </c>
       <c r="J2" s="41"/>
       <c r="K2" s="41"/>
@@ -8503,11 +8350,11 @@
       <c r="R2" s="41"/>
       <c r="S2" s="21">
         <f>SUM(Table1[[#This Row],[sep-25]:[Jun-26]])</f>
-        <v>9984</v>
+        <v>12756</v>
       </c>
       <c r="T2" s="19">
         <f t="shared" ref="T2:T11" si="0">IFERROR(S2/F2,0)</f>
-        <v>10.125760649087221</v>
+        <v>3.3943587014369347</v>
       </c>
       <c r="U2" s="14">
         <f>F2-S2</f>
@@ -9176,7 +9023,7 @@
     <row r="33" spans="10:10" ht="15.75" customHeight="1">
       <c r="J33">
         <f>SUM(G2:L2)</f>
-        <v>4883</v>
+        <v>7655</v>
       </c>
     </row>
   </sheetData>
@@ -9370,6 +9217,88 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{27A1C2DE-958E-4EF5-BD32-D7572A596892}">
+  <dimension ref="A1:C81"/>
+  <sheetFormatPr defaultColWidth="9" defaultRowHeight="16"/>
+  <sheetData>
+    <row r="1" spans="1:1">
+      <c r="A1" s="57">
+        <v>46062</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3">
+      <c r="A17">
+        <v>5911</v>
+      </c>
+      <c r="B17">
+        <v>3758</v>
+      </c>
+      <c r="C17" s="58">
+        <f>+B17/A17</f>
+        <v>0.63576383014718318</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3">
+      <c r="B18">
+        <v>986</v>
+      </c>
+      <c r="C18" s="58">
+        <f>+B18/A17</f>
+        <v>0.16680764676027746</v>
+      </c>
+    </row>
+    <row r="42" spans="1:1">
+      <c r="A42" s="57">
+        <v>46085</v>
+      </c>
+    </row>
+    <row r="69" spans="1:1">
+      <c r="A69" t="s">
+        <v>208</v>
+      </c>
+    </row>
+    <row r="70" spans="1:1">
+      <c r="A70">
+        <v>5943</v>
+      </c>
+    </row>
+    <row r="72" spans="1:1">
+      <c r="A72" t="s">
+        <v>209</v>
+      </c>
+    </row>
+    <row r="73" spans="1:1">
+      <c r="A73">
+        <v>5258</v>
+      </c>
+    </row>
+    <row r="75" spans="1:1">
+      <c r="A75" t="s">
+        <v>210</v>
+      </c>
+    </row>
+    <row r="76" spans="1:1">
+      <c r="A76">
+        <v>5101</v>
+      </c>
+    </row>
+    <row r="80" spans="1:1">
+      <c r="A80" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="81" spans="1:1">
+      <c r="A81">
+        <v>4884</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <drawing r:id="rId1"/>
+</worksheet>
+</file>
+
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
@@ -9382,15 +9311,6 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010067C3E934A0AA0B40A01BB34EE44DBE4E" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="99f90e1838b691a269ec0be7c9d3b1c4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7bc4fa38-d888-4f67-9acc-d35155363a39" xmlns:ns3="fff59cbe-7145-45c6-b0b8-a33a9ec94a75" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="55b527a863acd720578db25cd4da17b2" ns2:_="" ns3:_="">
     <xsd:import namespace="7bc4fa38-d888-4f67-9acc-d35155363a39"/>
@@ -9585,6 +9505,15 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9F09B98-3A3F-4A19-9439-839483AD047D}">
   <ds:schemaRefs>
@@ -9603,14 +9532,6 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57AD8670-20BC-4534-A7A5-87984349E00F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{339BB920-340D-4757-A55F-4B7C981C835F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9627,4 +9548,12 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57AD8670-20BC-4534-A7A5-87984349E00F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>

<commit_message>
feat(visuals): apply [Actual_Status] measure to KPI charts
Validated and applied the MAX date evaluation logic (filtering out pre-populated zeroes) to successfully retrieve the latest actual value. Updated dashboard visualizations to accurately reflect the current KPI progression.
</commit_message>
<xml_diff>
--- a/Datasets/okrs.xlsx
+++ b/Datasets/okrs.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauro.turner\Proyectos\Dashboards\Global-IT---OKR-KPI-Dashboard\Datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8331B162-FE24-49B7-8074-6047397F3554}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3B22E1-DA16-4099-B99A-3CF8BBA0C15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="810" firstSheet="1" activeTab="3" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="810" firstSheet="1" activeTab="7" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
   </bookViews>
   <sheets>
     <sheet name="objetives" sheetId="11" r:id="rId1"/>

</xml_diff>

<commit_message>
feat(ui, dax): add dynamic refresh timestamp to footer
Created [Last_Update_Text] measure extracting the max datetime from the 'updated_till' table. Formatted the output to standard corporate English ('Last updated: MMM DD, YYYY') to provide clear data freshness visibility to Global IT leadership.
</commit_message>
<xml_diff>
--- a/Datasets/okrs.xlsx
+++ b/Datasets/okrs.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29530"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29725"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mauro.turner\Proyectos\Dashboards\Global-IT---OKR-KPI-Dashboard\Datasets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DF3B22E1-DA16-4099-B99A-3CF8BBA0C15F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1D9DEAFB-B368-4EA9-B366-50167579845C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" tabRatio="810" firstSheet="1" activeTab="7" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
+    <workbookView xWindow="0" yWindow="760" windowWidth="19200" windowHeight="8570" tabRatio="810" firstSheet="1" activeTab="6" xr2:uid="{8E213388-CB59-1444-9D14-59F96BC33DF7}"/>
   </bookViews>
   <sheets>
     <sheet name="objetives" sheetId="11" r:id="rId1"/>
@@ -77,7 +77,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="543" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="554" uniqueCount="253">
   <si>
     <t>ID</t>
   </si>
@@ -1289,6 +1289,15 @@
   </si>
   <si>
     <t>Target_Unit</t>
+  </si>
+  <si>
+    <t>Tracking_Type</t>
+  </si>
+  <si>
+    <t>Cumulative</t>
+  </si>
+  <si>
+    <t>Snapshot</t>
   </si>
 </sst>
 </file>
@@ -3010,15 +3019,16 @@
 </file>
 
 <file path=xl/tables/table4.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{05CF7CEB-E38D-4385-9D0A-7780DBE1F2C6}" name="kpis" displayName="kpis" ref="A1:F11" totalsRowShown="0">
-  <autoFilter ref="A1:F11" xr:uid="{05CF7CEB-E38D-4385-9D0A-7780DBE1F2C6}"/>
-  <tableColumns count="6">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="9" xr:uid="{05CF7CEB-E38D-4385-9D0A-7780DBE1F2C6}" name="kpis" displayName="kpis" ref="A1:G11" totalsRowShown="0">
+  <autoFilter ref="A1:G11" xr:uid="{05CF7CEB-E38D-4385-9D0A-7780DBE1F2C6}"/>
+  <tableColumns count="7">
     <tableColumn id="1" xr3:uid="{68ECD000-5CB1-4C4B-BB03-A6A5B1FE144C}" name="KPI_ID"/>
     <tableColumn id="2" xr3:uid="{EE4E4C8E-E234-462A-B525-6959D9606CDE}" name="Objetive_ID"/>
     <tableColumn id="6" xr3:uid="{AC2714AF-A87A-4389-91F0-B64D137D4FCB}" name="Target_Unit"/>
     <tableColumn id="3" xr3:uid="{46D9FC96-8D58-4277-8E94-058CE19E84BF}" name="Actual_Unit"/>
     <tableColumn id="4" xr3:uid="{F5A9C9F6-F438-47DA-A6B5-34F34C02DBAD}" name="KPI_Goal"/>
     <tableColumn id="5" xr3:uid="{E5AD5A19-0EBD-4165-9D29-1E69182B7E49}" name="Target_Value"/>
+    <tableColumn id="7" xr3:uid="{D01E507C-3B3B-4D9D-A1DC-574FB15CB77A}" name="Tracking_Type"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -5424,7 +5434,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5716ADCC-E36E-44A5-AF6D-43063C282787}">
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:G11"/>
   <sheetFormatPr defaultColWidth="10.6640625" defaultRowHeight="16"/>
   <cols>
     <col min="2" max="3" width="12.08203125" customWidth="1"/>
@@ -5433,7 +5443,7 @@
     <col min="6" max="6" width="13.08203125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:7">
       <c r="A1" t="s">
         <v>214</v>
       </c>
@@ -5452,8 +5462,11 @@
       <c r="F1" t="s">
         <v>216</v>
       </c>
-    </row>
-    <row r="2" spans="1:6">
+      <c r="G1" t="s">
+        <v>250</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7">
       <c r="A2">
         <v>1</v>
       </c>
@@ -5472,8 +5485,11 @@
       <c r="F2">
         <v>0.2</v>
       </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="G2" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7">
       <c r="A3">
         <v>2</v>
       </c>
@@ -5492,8 +5508,11 @@
       <c r="F3">
         <v>0.7</v>
       </c>
-    </row>
-    <row r="4" spans="1:6">
+      <c r="G3" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7">
       <c r="A4">
         <v>3</v>
       </c>
@@ -5512,8 +5531,11 @@
       <c r="F4">
         <v>24</v>
       </c>
-    </row>
-    <row r="5" spans="1:6">
+      <c r="G4" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7">
       <c r="A5">
         <v>4</v>
       </c>
@@ -5532,8 +5554,11 @@
       <c r="F5">
         <v>2</v>
       </c>
-    </row>
-    <row r="6" spans="1:6">
+      <c r="G5" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7">
       <c r="A6">
         <v>5</v>
       </c>
@@ -5552,8 +5577,11 @@
       <c r="F6">
         <v>30</v>
       </c>
-    </row>
-    <row r="7" spans="1:6">
+      <c r="G6" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7">
       <c r="A7">
         <v>6</v>
       </c>
@@ -5572,8 +5600,11 @@
       <c r="F7">
         <v>10</v>
       </c>
-    </row>
-    <row r="8" spans="1:6">
+      <c r="G7" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7">
       <c r="A8">
         <v>7</v>
       </c>
@@ -5592,8 +5623,11 @@
       <c r="F8">
         <v>4</v>
       </c>
-    </row>
-    <row r="9" spans="1:6">
+      <c r="G8" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7">
       <c r="A9">
         <v>8</v>
       </c>
@@ -5612,8 +5646,11 @@
       <c r="F9">
         <v>1</v>
       </c>
-    </row>
-    <row r="10" spans="1:6">
+      <c r="G9" t="s">
+        <v>252</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7">
       <c r="A10">
         <v>9</v>
       </c>
@@ -5632,8 +5669,11 @@
       <c r="F10">
         <v>3</v>
       </c>
-    </row>
-    <row r="11" spans="1:6">
+      <c r="G10" t="s">
+        <v>251</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7">
       <c r="A11">
         <v>10</v>
       </c>
@@ -5642,6 +5682,9 @@
       </c>
       <c r="E11" t="s">
         <v>31</v>
+      </c>
+      <c r="G11" t="s">
+        <v>251</v>
       </c>
     </row>
   </sheetData>
@@ -7647,7 +7690,7 @@
         <v>46082</v>
       </c>
       <c r="D92">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="E92" t="s">
         <v>246</v>
@@ -8798,7 +8841,7 @@
         <v>0.8</v>
       </c>
       <c r="M9" s="44">
-        <v>1</v>
+        <v>0.9</v>
       </c>
       <c r="N9" s="44">
         <v>0</v>
@@ -8817,15 +8860,15 @@
       </c>
       <c r="S9" s="21">
         <f>SUM(G9:R9)</f>
-        <v>5.8</v>
+        <v>5.7</v>
       </c>
       <c r="T9" s="22">
         <f t="shared" si="0"/>
-        <v>7.2499999999999991</v>
+        <v>7.125</v>
       </c>
       <c r="U9" s="23">
         <f t="shared" ref="U9:U10" si="2">F9-S9</f>
-        <v>-5</v>
+        <v>-4.9000000000000004</v>
       </c>
       <c r="V9" s="18"/>
     </row>
@@ -9311,6 +9354,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x01010067C3E934A0AA0B40A01BB34EE44DBE4E" ma:contentTypeVersion="11" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="99f90e1838b691a269ec0be7c9d3b1c4">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="7bc4fa38-d888-4f67-9acc-d35155363a39" xmlns:ns3="fff59cbe-7145-45c6-b0b8-a33a9ec94a75" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="55b527a863acd720578db25cd4da17b2" ns2:_="" ns3:_="">
     <xsd:import namespace="7bc4fa38-d888-4f67-9acc-d35155363a39"/>
@@ -9505,15 +9557,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F9F09B98-3A3F-4A19-9439-839483AD047D}">
   <ds:schemaRefs>
@@ -9532,6 +9575,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57AD8670-20BC-4534-A7A5-87984349E00F}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{339BB920-340D-4757-A55F-4B7C981C835F}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -9548,12 +9599,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{57AD8670-20BC-4534-A7A5-87984349E00F}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>